<commit_message>
update report external quality - new spec V2.1
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportExternalQualityReportTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportExternalQualityReportTemplate.xlsx
@@ -1,17 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Clone\23-kcvn-spm-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Báo cáo KTTN và Xuất Hàng" sheetId="1" r:id="rId4"/>
+    <sheet name="Báo cáo KTTN và Xuất Hàng" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>Tên rút gọn</t>
   </si>
@@ -58,28 +66,28 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Microsoft YaHei"/>
     </font>
@@ -89,42 +97,51 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -314,30 +331,31 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AA1000"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="14.0"/>
-    <col customWidth="1" min="2" max="2" width="18.0"/>
-    <col customWidth="1" min="3" max="3" width="19.0"/>
-    <col customWidth="1" min="4" max="4" width="18.75"/>
-    <col customWidth="1" min="5" max="6" width="12.63"/>
-    <col customWidth="1" min="7" max="7" width="14.25"/>
-    <col customWidth="1" min="8" max="8" width="16.25"/>
-    <col customWidth="1" min="10" max="10" width="19.88"/>
-    <col customWidth="1" min="12" max="12" width="42.63"/>
-    <col customWidth="1" min="13" max="13" width="38.25"/>
-    <col customWidth="1" min="14" max="14" width="10.25"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="6" width="12.5703125" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" customWidth="1"/>
+    <col min="8" max="8" width="16.28515625" customWidth="1"/>
+    <col min="10" max="10" width="19.85546875" customWidth="1"/>
+    <col min="12" max="12" width="23.5703125" customWidth="1"/>
+    <col min="13" max="13" width="42.5703125" customWidth="1"/>
+    <col min="14" max="14" width="38.28515625" customWidth="1"/>
+    <col min="15" max="15" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="23.25" customHeight="1">
+    <row r="1" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -364,8 +382,9 @@
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
-    </row>
-    <row r="2" ht="27.75" customHeight="1">
+      <c r="AA1" s="1"/>
+    </row>
+    <row r="2" spans="1:27" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -400,15 +419,17 @@
         <v>10</v>
       </c>
       <c r="L2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="1"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -420,8 +441,9 @@
       <c r="X2" s="1"/>
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
-    </row>
-    <row r="3" ht="15.75" customHeight="1">
+      <c r="AA2" s="1"/>
+    </row>
+    <row r="3" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -448,8 +470,9 @@
       <c r="X3" s="1"/>
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
-    </row>
-    <row r="4" ht="15.75" customHeight="1">
+      <c r="AA3" s="1"/>
+    </row>
+    <row r="4" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -476,8 +499,9 @@
       <c r="X4" s="1"/>
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
-    </row>
-    <row r="5" ht="15.75" customHeight="1">
+      <c r="AA4" s="1"/>
+    </row>
+    <row r="5" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -504,8 +528,9 @@
       <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
-    </row>
-    <row r="6" ht="15.75" customHeight="1">
+      <c r="AA5" s="1"/>
+    </row>
+    <row r="6" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -532,8 +557,9 @@
       <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
-    </row>
-    <row r="7" ht="15.75" customHeight="1">
+      <c r="AA6" s="1"/>
+    </row>
+    <row r="7" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -560,8 +586,9 @@
       <c r="X7" s="1"/>
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
-    </row>
-    <row r="8" ht="15.75" customHeight="1">
+      <c r="AA7" s="1"/>
+    </row>
+    <row r="8" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -588,8 +615,9 @@
       <c r="X8" s="1"/>
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
-    </row>
-    <row r="9" ht="15.75" customHeight="1">
+      <c r="AA8" s="1"/>
+    </row>
+    <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -616,8 +644,9 @@
       <c r="X9" s="1"/>
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
-    </row>
-    <row r="10" ht="15.75" customHeight="1">
+      <c r="AA9" s="1"/>
+    </row>
+    <row r="10" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -644,8 +673,9 @@
       <c r="X10" s="1"/>
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
-    </row>
-    <row r="11" ht="15.75" customHeight="1">
+      <c r="AA10" s="1"/>
+    </row>
+    <row r="11" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -672,8 +702,9 @@
       <c r="X11" s="1"/>
       <c r="Y11" s="1"/>
       <c r="Z11" s="1"/>
-    </row>
-    <row r="12" ht="15.75" customHeight="1">
+      <c r="AA11" s="1"/>
+    </row>
+    <row r="12" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -700,8 +731,9 @@
       <c r="X12" s="1"/>
       <c r="Y12" s="1"/>
       <c r="Z12" s="1"/>
-    </row>
-    <row r="13" ht="15.75" customHeight="1">
+      <c r="AA12" s="1"/>
+    </row>
+    <row r="13" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -728,8 +760,9 @@
       <c r="X13" s="1"/>
       <c r="Y13" s="1"/>
       <c r="Z13" s="1"/>
-    </row>
-    <row r="14" ht="15.75" customHeight="1">
+      <c r="AA13" s="1"/>
+    </row>
+    <row r="14" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -756,8 +789,9 @@
       <c r="X14" s="1"/>
       <c r="Y14" s="1"/>
       <c r="Z14" s="1"/>
-    </row>
-    <row r="15" ht="15.75" customHeight="1">
+      <c r="AA14" s="1"/>
+    </row>
+    <row r="15" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -784,8 +818,9 @@
       <c r="X15" s="1"/>
       <c r="Y15" s="1"/>
       <c r="Z15" s="1"/>
-    </row>
-    <row r="16" ht="15.75" customHeight="1">
+      <c r="AA15" s="1"/>
+    </row>
+    <row r="16" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -812,8 +847,9 @@
       <c r="X16" s="1"/>
       <c r="Y16" s="1"/>
       <c r="Z16" s="1"/>
-    </row>
-    <row r="17" ht="15.75" customHeight="1">
+      <c r="AA16" s="1"/>
+    </row>
+    <row r="17" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -840,8 +876,9 @@
       <c r="X17" s="1"/>
       <c r="Y17" s="1"/>
       <c r="Z17" s="1"/>
-    </row>
-    <row r="18" ht="15.75" customHeight="1">
+      <c r="AA17" s="1"/>
+    </row>
+    <row r="18" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -868,8 +905,9 @@
       <c r="X18" s="1"/>
       <c r="Y18" s="1"/>
       <c r="Z18" s="1"/>
-    </row>
-    <row r="19" ht="15.75" customHeight="1">
+      <c r="AA18" s="1"/>
+    </row>
+    <row r="19" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -896,8 +934,9 @@
       <c r="X19" s="1"/>
       <c r="Y19" s="1"/>
       <c r="Z19" s="1"/>
-    </row>
-    <row r="20" ht="15.75" customHeight="1">
+      <c r="AA19" s="1"/>
+    </row>
+    <row r="20" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -924,8 +963,9 @@
       <c r="X20" s="1"/>
       <c r="Y20" s="1"/>
       <c r="Z20" s="1"/>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
+      <c r="AA20" s="1"/>
+    </row>
+    <row r="21" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -952,8 +992,9 @@
       <c r="X21" s="1"/>
       <c r="Y21" s="1"/>
       <c r="Z21" s="1"/>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
+      <c r="AA21" s="1"/>
+    </row>
+    <row r="22" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -980,8 +1021,9 @@
       <c r="X22" s="1"/>
       <c r="Y22" s="1"/>
       <c r="Z22" s="1"/>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
+      <c r="AA22" s="1"/>
+    </row>
+    <row r="23" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1008,8 +1050,9 @@
       <c r="X23" s="1"/>
       <c r="Y23" s="1"/>
       <c r="Z23" s="1"/>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
+      <c r="AA23" s="1"/>
+    </row>
+    <row r="24" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1036,8 +1079,9 @@
       <c r="X24" s="1"/>
       <c r="Y24" s="1"/>
       <c r="Z24" s="1"/>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
+      <c r="AA24" s="1"/>
+    </row>
+    <row r="25" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1064,8 +1108,9 @@
       <c r="X25" s="1"/>
       <c r="Y25" s="1"/>
       <c r="Z25" s="1"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
+      <c r="AA25" s="1"/>
+    </row>
+    <row r="26" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1092,8 +1137,9 @@
       <c r="X26" s="1"/>
       <c r="Y26" s="1"/>
       <c r="Z26" s="1"/>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
+      <c r="AA26" s="1"/>
+    </row>
+    <row r="27" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1120,8 +1166,9 @@
       <c r="X27" s="1"/>
       <c r="Y27" s="1"/>
       <c r="Z27" s="1"/>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
+      <c r="AA27" s="1"/>
+    </row>
+    <row r="28" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1148,8 +1195,9 @@
       <c r="X28" s="1"/>
       <c r="Y28" s="1"/>
       <c r="Z28" s="1"/>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
+      <c r="AA28" s="1"/>
+    </row>
+    <row r="29" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1176,8 +1224,9 @@
       <c r="X29" s="1"/>
       <c r="Y29" s="1"/>
       <c r="Z29" s="1"/>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
+      <c r="AA29" s="1"/>
+    </row>
+    <row r="30" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -1204,8 +1253,9 @@
       <c r="X30" s="1"/>
       <c r="Y30" s="1"/>
       <c r="Z30" s="1"/>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
+      <c r="AA30" s="1"/>
+    </row>
+    <row r="31" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1232,8 +1282,9 @@
       <c r="X31" s="1"/>
       <c r="Y31" s="1"/>
       <c r="Z31" s="1"/>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
+      <c r="AA31" s="1"/>
+    </row>
+    <row r="32" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -1260,8 +1311,9 @@
       <c r="X32" s="1"/>
       <c r="Y32" s="1"/>
       <c r="Z32" s="1"/>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
+      <c r="AA32" s="1"/>
+    </row>
+    <row r="33" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -1288,8 +1340,9 @@
       <c r="X33" s="1"/>
       <c r="Y33" s="1"/>
       <c r="Z33" s="1"/>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
+      <c r="AA33" s="1"/>
+    </row>
+    <row r="34" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -1316,8 +1369,9 @@
       <c r="X34" s="1"/>
       <c r="Y34" s="1"/>
       <c r="Z34" s="1"/>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
+      <c r="AA34" s="1"/>
+    </row>
+    <row r="35" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -1344,8 +1398,9 @@
       <c r="X35" s="1"/>
       <c r="Y35" s="1"/>
       <c r="Z35" s="1"/>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
+      <c r="AA35" s="1"/>
+    </row>
+    <row r="36" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -1372,8 +1427,9 @@
       <c r="X36" s="1"/>
       <c r="Y36" s="1"/>
       <c r="Z36" s="1"/>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
+      <c r="AA36" s="1"/>
+    </row>
+    <row r="37" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -1400,8 +1456,9 @@
       <c r="X37" s="1"/>
       <c r="Y37" s="1"/>
       <c r="Z37" s="1"/>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
+      <c r="AA37" s="1"/>
+    </row>
+    <row r="38" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -1428,8 +1485,9 @@
       <c r="X38" s="1"/>
       <c r="Y38" s="1"/>
       <c r="Z38" s="1"/>
-    </row>
-    <row r="39" ht="15.75" customHeight="1">
+      <c r="AA38" s="1"/>
+    </row>
+    <row r="39" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -1456,8 +1514,9 @@
       <c r="X39" s="1"/>
       <c r="Y39" s="1"/>
       <c r="Z39" s="1"/>
-    </row>
-    <row r="40" ht="15.75" customHeight="1">
+      <c r="AA39" s="1"/>
+    </row>
+    <row r="40" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -1484,8 +1543,9 @@
       <c r="X40" s="1"/>
       <c r="Y40" s="1"/>
       <c r="Z40" s="1"/>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
+      <c r="AA40" s="1"/>
+    </row>
+    <row r="41" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -1512,8 +1572,9 @@
       <c r="X41" s="1"/>
       <c r="Y41" s="1"/>
       <c r="Z41" s="1"/>
-    </row>
-    <row r="42" ht="15.75" customHeight="1">
+      <c r="AA41" s="1"/>
+    </row>
+    <row r="42" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -1540,8 +1601,9 @@
       <c r="X42" s="1"/>
       <c r="Y42" s="1"/>
       <c r="Z42" s="1"/>
-    </row>
-    <row r="43" ht="15.75" customHeight="1">
+      <c r="AA42" s="1"/>
+    </row>
+    <row r="43" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -1568,8 +1630,9 @@
       <c r="X43" s="1"/>
       <c r="Y43" s="1"/>
       <c r="Z43" s="1"/>
-    </row>
-    <row r="44" ht="15.75" customHeight="1">
+      <c r="AA43" s="1"/>
+    </row>
+    <row r="44" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -1596,8 +1659,9 @@
       <c r="X44" s="1"/>
       <c r="Y44" s="1"/>
       <c r="Z44" s="1"/>
-    </row>
-    <row r="45" ht="15.75" customHeight="1">
+      <c r="AA44" s="1"/>
+    </row>
+    <row r="45" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -1624,8 +1688,9 @@
       <c r="X45" s="1"/>
       <c r="Y45" s="1"/>
       <c r="Z45" s="1"/>
-    </row>
-    <row r="46" ht="15.75" customHeight="1">
+      <c r="AA45" s="1"/>
+    </row>
+    <row r="46" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -1652,8 +1717,9 @@
       <c r="X46" s="1"/>
       <c r="Y46" s="1"/>
       <c r="Z46" s="1"/>
-    </row>
-    <row r="47" ht="15.75" customHeight="1">
+      <c r="AA46" s="1"/>
+    </row>
+    <row r="47" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -1680,8 +1746,9 @@
       <c r="X47" s="1"/>
       <c r="Y47" s="1"/>
       <c r="Z47" s="1"/>
-    </row>
-    <row r="48" ht="15.75" customHeight="1">
+      <c r="AA47" s="1"/>
+    </row>
+    <row r="48" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -1708,8 +1775,9 @@
       <c r="X48" s="1"/>
       <c r="Y48" s="1"/>
       <c r="Z48" s="1"/>
-    </row>
-    <row r="49" ht="15.75" customHeight="1">
+      <c r="AA48" s="1"/>
+    </row>
+    <row r="49" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -1736,8 +1804,9 @@
       <c r="X49" s="1"/>
       <c r="Y49" s="1"/>
       <c r="Z49" s="1"/>
-    </row>
-    <row r="50" ht="15.75" customHeight="1">
+      <c r="AA49" s="1"/>
+    </row>
+    <row r="50" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -1764,8 +1833,9 @@
       <c r="X50" s="1"/>
       <c r="Y50" s="1"/>
       <c r="Z50" s="1"/>
-    </row>
-    <row r="51" ht="15.75" customHeight="1">
+      <c r="AA50" s="1"/>
+    </row>
+    <row r="51" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -1792,8 +1862,9 @@
       <c r="X51" s="1"/>
       <c r="Y51" s="1"/>
       <c r="Z51" s="1"/>
-    </row>
-    <row r="52" ht="15.75" customHeight="1">
+      <c r="AA51" s="1"/>
+    </row>
+    <row r="52" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -1820,8 +1891,9 @@
       <c r="X52" s="1"/>
       <c r="Y52" s="1"/>
       <c r="Z52" s="1"/>
-    </row>
-    <row r="53" ht="15.75" customHeight="1">
+      <c r="AA52" s="1"/>
+    </row>
+    <row r="53" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -1848,8 +1920,9 @@
       <c r="X53" s="1"/>
       <c r="Y53" s="1"/>
       <c r="Z53" s="1"/>
-    </row>
-    <row r="54" ht="15.75" customHeight="1">
+      <c r="AA53" s="1"/>
+    </row>
+    <row r="54" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -1876,8 +1949,9 @@
       <c r="X54" s="1"/>
       <c r="Y54" s="1"/>
       <c r="Z54" s="1"/>
-    </row>
-    <row r="55" ht="15.75" customHeight="1">
+      <c r="AA54" s="1"/>
+    </row>
+    <row r="55" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -1904,8 +1978,9 @@
       <c r="X55" s="1"/>
       <c r="Y55" s="1"/>
       <c r="Z55" s="1"/>
-    </row>
-    <row r="56" ht="15.75" customHeight="1">
+      <c r="AA55" s="1"/>
+    </row>
+    <row r="56" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -1932,8 +2007,9 @@
       <c r="X56" s="1"/>
       <c r="Y56" s="1"/>
       <c r="Z56" s="1"/>
-    </row>
-    <row r="57" ht="15.75" customHeight="1">
+      <c r="AA56" s="1"/>
+    </row>
+    <row r="57" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -1960,8 +2036,9 @@
       <c r="X57" s="1"/>
       <c r="Y57" s="1"/>
       <c r="Z57" s="1"/>
-    </row>
-    <row r="58" ht="15.75" customHeight="1">
+      <c r="AA57" s="1"/>
+    </row>
+    <row r="58" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -1988,8 +2065,9 @@
       <c r="X58" s="1"/>
       <c r="Y58" s="1"/>
       <c r="Z58" s="1"/>
-    </row>
-    <row r="59" ht="15.75" customHeight="1">
+      <c r="AA58" s="1"/>
+    </row>
+    <row r="59" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -2016,8 +2094,9 @@
       <c r="X59" s="1"/>
       <c r="Y59" s="1"/>
       <c r="Z59" s="1"/>
-    </row>
-    <row r="60" ht="15.75" customHeight="1">
+      <c r="AA59" s="1"/>
+    </row>
+    <row r="60" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -2044,8 +2123,9 @@
       <c r="X60" s="1"/>
       <c r="Y60" s="1"/>
       <c r="Z60" s="1"/>
-    </row>
-    <row r="61" ht="15.75" customHeight="1">
+      <c r="AA60" s="1"/>
+    </row>
+    <row r="61" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -2072,8 +2152,9 @@
       <c r="X61" s="1"/>
       <c r="Y61" s="1"/>
       <c r="Z61" s="1"/>
-    </row>
-    <row r="62" ht="15.75" customHeight="1">
+      <c r="AA61" s="1"/>
+    </row>
+    <row r="62" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
@@ -2100,8 +2181,9 @@
       <c r="X62" s="1"/>
       <c r="Y62" s="1"/>
       <c r="Z62" s="1"/>
-    </row>
-    <row r="63" ht="15.75" customHeight="1">
+      <c r="AA62" s="1"/>
+    </row>
+    <row r="63" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
@@ -2128,8 +2210,9 @@
       <c r="X63" s="1"/>
       <c r="Y63" s="1"/>
       <c r="Z63" s="1"/>
-    </row>
-    <row r="64" ht="15.75" customHeight="1">
+      <c r="AA63" s="1"/>
+    </row>
+    <row r="64" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
@@ -2156,8 +2239,9 @@
       <c r="X64" s="1"/>
       <c r="Y64" s="1"/>
       <c r="Z64" s="1"/>
-    </row>
-    <row r="65" ht="15.75" customHeight="1">
+      <c r="AA64" s="1"/>
+    </row>
+    <row r="65" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
@@ -2184,8 +2268,9 @@
       <c r="X65" s="1"/>
       <c r="Y65" s="1"/>
       <c r="Z65" s="1"/>
-    </row>
-    <row r="66" ht="15.75" customHeight="1">
+      <c r="AA65" s="1"/>
+    </row>
+    <row r="66" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
@@ -2212,8 +2297,9 @@
       <c r="X66" s="1"/>
       <c r="Y66" s="1"/>
       <c r="Z66" s="1"/>
-    </row>
-    <row r="67" ht="15.75" customHeight="1">
+      <c r="AA66" s="1"/>
+    </row>
+    <row r="67" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -2240,8 +2326,9 @@
       <c r="X67" s="1"/>
       <c r="Y67" s="1"/>
       <c r="Z67" s="1"/>
-    </row>
-    <row r="68" ht="15.75" customHeight="1">
+      <c r="AA67" s="1"/>
+    </row>
+    <row r="68" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -2268,8 +2355,9 @@
       <c r="X68" s="1"/>
       <c r="Y68" s="1"/>
       <c r="Z68" s="1"/>
-    </row>
-    <row r="69" ht="15.75" customHeight="1">
+      <c r="AA68" s="1"/>
+    </row>
+    <row r="69" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
@@ -2296,8 +2384,9 @@
       <c r="X69" s="1"/>
       <c r="Y69" s="1"/>
       <c r="Z69" s="1"/>
-    </row>
-    <row r="70" ht="15.75" customHeight="1">
+      <c r="AA69" s="1"/>
+    </row>
+    <row r="70" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
@@ -2324,8 +2413,9 @@
       <c r="X70" s="1"/>
       <c r="Y70" s="1"/>
       <c r="Z70" s="1"/>
-    </row>
-    <row r="71" ht="15.75" customHeight="1">
+      <c r="AA70" s="1"/>
+    </row>
+    <row r="71" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
@@ -2352,8 +2442,9 @@
       <c r="X71" s="1"/>
       <c r="Y71" s="1"/>
       <c r="Z71" s="1"/>
-    </row>
-    <row r="72" ht="15.75" customHeight="1">
+      <c r="AA71" s="1"/>
+    </row>
+    <row r="72" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
@@ -2380,8 +2471,9 @@
       <c r="X72" s="1"/>
       <c r="Y72" s="1"/>
       <c r="Z72" s="1"/>
-    </row>
-    <row r="73" ht="15.75" customHeight="1">
+      <c r="AA72" s="1"/>
+    </row>
+    <row r="73" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
@@ -2408,8 +2500,9 @@
       <c r="X73" s="1"/>
       <c r="Y73" s="1"/>
       <c r="Z73" s="1"/>
-    </row>
-    <row r="74" ht="15.75" customHeight="1">
+      <c r="AA73" s="1"/>
+    </row>
+    <row r="74" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
@@ -2436,8 +2529,9 @@
       <c r="X74" s="1"/>
       <c r="Y74" s="1"/>
       <c r="Z74" s="1"/>
-    </row>
-    <row r="75" ht="15.75" customHeight="1">
+      <c r="AA74" s="1"/>
+    </row>
+    <row r="75" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
@@ -2464,8 +2558,9 @@
       <c r="X75" s="1"/>
       <c r="Y75" s="1"/>
       <c r="Z75" s="1"/>
-    </row>
-    <row r="76" ht="15.75" customHeight="1">
+      <c r="AA75" s="1"/>
+    </row>
+    <row r="76" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
@@ -2492,8 +2587,9 @@
       <c r="X76" s="1"/>
       <c r="Y76" s="1"/>
       <c r="Z76" s="1"/>
-    </row>
-    <row r="77" ht="15.75" customHeight="1">
+      <c r="AA76" s="1"/>
+    </row>
+    <row r="77" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
@@ -2520,8 +2616,9 @@
       <c r="X77" s="1"/>
       <c r="Y77" s="1"/>
       <c r="Z77" s="1"/>
-    </row>
-    <row r="78" ht="15.75" customHeight="1">
+      <c r="AA77" s="1"/>
+    </row>
+    <row r="78" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
@@ -2548,8 +2645,9 @@
       <c r="X78" s="1"/>
       <c r="Y78" s="1"/>
       <c r="Z78" s="1"/>
-    </row>
-    <row r="79" ht="15.75" customHeight="1">
+      <c r="AA78" s="1"/>
+    </row>
+    <row r="79" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -2576,8 +2674,9 @@
       <c r="X79" s="1"/>
       <c r="Y79" s="1"/>
       <c r="Z79" s="1"/>
-    </row>
-    <row r="80" ht="15.75" customHeight="1">
+      <c r="AA79" s="1"/>
+    </row>
+    <row r="80" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
@@ -2604,8 +2703,9 @@
       <c r="X80" s="1"/>
       <c r="Y80" s="1"/>
       <c r="Z80" s="1"/>
-    </row>
-    <row r="81" ht="15.75" customHeight="1">
+      <c r="AA80" s="1"/>
+    </row>
+    <row r="81" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
@@ -2632,8 +2732,9 @@
       <c r="X81" s="1"/>
       <c r="Y81" s="1"/>
       <c r="Z81" s="1"/>
-    </row>
-    <row r="82" ht="15.75" customHeight="1">
+      <c r="AA81" s="1"/>
+    </row>
+    <row r="82" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -2660,8 +2761,9 @@
       <c r="X82" s="1"/>
       <c r="Y82" s="1"/>
       <c r="Z82" s="1"/>
-    </row>
-    <row r="83" ht="15.75" customHeight="1">
+      <c r="AA82" s="1"/>
+    </row>
+    <row r="83" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
@@ -2688,8 +2790,9 @@
       <c r="X83" s="1"/>
       <c r="Y83" s="1"/>
       <c r="Z83" s="1"/>
-    </row>
-    <row r="84" ht="15.75" customHeight="1">
+      <c r="AA83" s="1"/>
+    </row>
+    <row r="84" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -2716,8 +2819,9 @@
       <c r="X84" s="1"/>
       <c r="Y84" s="1"/>
       <c r="Z84" s="1"/>
-    </row>
-    <row r="85" ht="15.75" customHeight="1">
+      <c r="AA84" s="1"/>
+    </row>
+    <row r="85" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
@@ -2744,8 +2848,9 @@
       <c r="X85" s="1"/>
       <c r="Y85" s="1"/>
       <c r="Z85" s="1"/>
-    </row>
-    <row r="86" ht="15.75" customHeight="1">
+      <c r="AA85" s="1"/>
+    </row>
+    <row r="86" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
@@ -2772,8 +2877,9 @@
       <c r="X86" s="1"/>
       <c r="Y86" s="1"/>
       <c r="Z86" s="1"/>
-    </row>
-    <row r="87" ht="15.75" customHeight="1">
+      <c r="AA86" s="1"/>
+    </row>
+    <row r="87" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
@@ -2800,8 +2906,9 @@
       <c r="X87" s="1"/>
       <c r="Y87" s="1"/>
       <c r="Z87" s="1"/>
-    </row>
-    <row r="88" ht="15.75" customHeight="1">
+      <c r="AA87" s="1"/>
+    </row>
+    <row r="88" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
@@ -2828,8 +2935,9 @@
       <c r="X88" s="1"/>
       <c r="Y88" s="1"/>
       <c r="Z88" s="1"/>
-    </row>
-    <row r="89" ht="15.75" customHeight="1">
+      <c r="AA88" s="1"/>
+    </row>
+    <row r="89" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
@@ -2856,8 +2964,9 @@
       <c r="X89" s="1"/>
       <c r="Y89" s="1"/>
       <c r="Z89" s="1"/>
-    </row>
-    <row r="90" ht="15.75" customHeight="1">
+      <c r="AA89" s="1"/>
+    </row>
+    <row r="90" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
@@ -2884,8 +2993,9 @@
       <c r="X90" s="1"/>
       <c r="Y90" s="1"/>
       <c r="Z90" s="1"/>
-    </row>
-    <row r="91" ht="15.75" customHeight="1">
+      <c r="AA90" s="1"/>
+    </row>
+    <row r="91" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
@@ -2912,8 +3022,9 @@
       <c r="X91" s="1"/>
       <c r="Y91" s="1"/>
       <c r="Z91" s="1"/>
-    </row>
-    <row r="92" ht="15.75" customHeight="1">
+      <c r="AA91" s="1"/>
+    </row>
+    <row r="92" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
@@ -2940,8 +3051,9 @@
       <c r="X92" s="1"/>
       <c r="Y92" s="1"/>
       <c r="Z92" s="1"/>
-    </row>
-    <row r="93" ht="15.75" customHeight="1">
+      <c r="AA92" s="1"/>
+    </row>
+    <row r="93" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
@@ -2968,8 +3080,9 @@
       <c r="X93" s="1"/>
       <c r="Y93" s="1"/>
       <c r="Z93" s="1"/>
-    </row>
-    <row r="94" ht="15.75" customHeight="1">
+      <c r="AA93" s="1"/>
+    </row>
+    <row r="94" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
@@ -2996,8 +3109,9 @@
       <c r="X94" s="1"/>
       <c r="Y94" s="1"/>
       <c r="Z94" s="1"/>
-    </row>
-    <row r="95" ht="15.75" customHeight="1">
+      <c r="AA94" s="1"/>
+    </row>
+    <row r="95" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
@@ -3024,8 +3138,9 @@
       <c r="X95" s="1"/>
       <c r="Y95" s="1"/>
       <c r="Z95" s="1"/>
-    </row>
-    <row r="96" ht="15.75" customHeight="1">
+      <c r="AA95" s="1"/>
+    </row>
+    <row r="96" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
@@ -3052,8 +3167,9 @@
       <c r="X96" s="1"/>
       <c r="Y96" s="1"/>
       <c r="Z96" s="1"/>
-    </row>
-    <row r="97" ht="15.75" customHeight="1">
+      <c r="AA96" s="1"/>
+    </row>
+    <row r="97" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
@@ -3080,8 +3196,9 @@
       <c r="X97" s="1"/>
       <c r="Y97" s="1"/>
       <c r="Z97" s="1"/>
-    </row>
-    <row r="98" ht="15.75" customHeight="1">
+      <c r="AA97" s="1"/>
+    </row>
+    <row r="98" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
@@ -3108,8 +3225,9 @@
       <c r="X98" s="1"/>
       <c r="Y98" s="1"/>
       <c r="Z98" s="1"/>
-    </row>
-    <row r="99" ht="15.75" customHeight="1">
+      <c r="AA98" s="1"/>
+    </row>
+    <row r="99" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="1"/>
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
@@ -3136,8 +3254,9 @@
       <c r="X99" s="1"/>
       <c r="Y99" s="1"/>
       <c r="Z99" s="1"/>
-    </row>
-    <row r="100" ht="15.75" customHeight="1">
+      <c r="AA99" s="1"/>
+    </row>
+    <row r="100" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="1"/>
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
@@ -3164,8 +3283,9 @@
       <c r="X100" s="1"/>
       <c r="Y100" s="1"/>
       <c r="Z100" s="1"/>
-    </row>
-    <row r="101" ht="15.75" customHeight="1">
+      <c r="AA100" s="1"/>
+    </row>
+    <row r="101" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="1"/>
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
@@ -3192,8 +3312,9 @@
       <c r="X101" s="1"/>
       <c r="Y101" s="1"/>
       <c r="Z101" s="1"/>
-    </row>
-    <row r="102" ht="15.75" customHeight="1">
+      <c r="AA101" s="1"/>
+    </row>
+    <row r="102" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="1"/>
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
@@ -3220,8 +3341,9 @@
       <c r="X102" s="1"/>
       <c r="Y102" s="1"/>
       <c r="Z102" s="1"/>
-    </row>
-    <row r="103" ht="15.75" customHeight="1">
+      <c r="AA102" s="1"/>
+    </row>
+    <row r="103" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
@@ -3248,8 +3370,9 @@
       <c r="X103" s="1"/>
       <c r="Y103" s="1"/>
       <c r="Z103" s="1"/>
-    </row>
-    <row r="104" ht="15.75" customHeight="1">
+      <c r="AA103" s="1"/>
+    </row>
+    <row r="104" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -3276,8 +3399,9 @@
       <c r="X104" s="1"/>
       <c r="Y104" s="1"/>
       <c r="Z104" s="1"/>
-    </row>
-    <row r="105" ht="15.75" customHeight="1">
+      <c r="AA104" s="1"/>
+    </row>
+    <row r="105" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="1"/>
       <c r="B105" s="1"/>
       <c r="C105" s="1"/>
@@ -3304,8 +3428,9 @@
       <c r="X105" s="1"/>
       <c r="Y105" s="1"/>
       <c r="Z105" s="1"/>
-    </row>
-    <row r="106" ht="15.75" customHeight="1">
+      <c r="AA105" s="1"/>
+    </row>
+    <row r="106" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="1"/>
       <c r="B106" s="1"/>
       <c r="C106" s="1"/>
@@ -3332,8 +3457,9 @@
       <c r="X106" s="1"/>
       <c r="Y106" s="1"/>
       <c r="Z106" s="1"/>
-    </row>
-    <row r="107" ht="15.75" customHeight="1">
+      <c r="AA106" s="1"/>
+    </row>
+    <row r="107" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="1"/>
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
@@ -3360,8 +3486,9 @@
       <c r="X107" s="1"/>
       <c r="Y107" s="1"/>
       <c r="Z107" s="1"/>
-    </row>
-    <row r="108" ht="15.75" customHeight="1">
+      <c r="AA107" s="1"/>
+    </row>
+    <row r="108" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="1"/>
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
@@ -3388,8 +3515,9 @@
       <c r="X108" s="1"/>
       <c r="Y108" s="1"/>
       <c r="Z108" s="1"/>
-    </row>
-    <row r="109" ht="15.75" customHeight="1">
+      <c r="AA108" s="1"/>
+    </row>
+    <row r="109" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="1"/>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
@@ -3416,8 +3544,9 @@
       <c r="X109" s="1"/>
       <c r="Y109" s="1"/>
       <c r="Z109" s="1"/>
-    </row>
-    <row r="110" ht="15.75" customHeight="1">
+      <c r="AA109" s="1"/>
+    </row>
+    <row r="110" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -3444,8 +3573,9 @@
       <c r="X110" s="1"/>
       <c r="Y110" s="1"/>
       <c r="Z110" s="1"/>
-    </row>
-    <row r="111" ht="15.75" customHeight="1">
+      <c r="AA110" s="1"/>
+    </row>
+    <row r="111" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="1"/>
       <c r="B111" s="1"/>
       <c r="C111" s="1"/>
@@ -3472,8 +3602,9 @@
       <c r="X111" s="1"/>
       <c r="Y111" s="1"/>
       <c r="Z111" s="1"/>
-    </row>
-    <row r="112" ht="15.75" customHeight="1">
+      <c r="AA111" s="1"/>
+    </row>
+    <row r="112" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="1"/>
       <c r="B112" s="1"/>
       <c r="C112" s="1"/>
@@ -3500,8 +3631,9 @@
       <c r="X112" s="1"/>
       <c r="Y112" s="1"/>
       <c r="Z112" s="1"/>
-    </row>
-    <row r="113" ht="15.75" customHeight="1">
+      <c r="AA112" s="1"/>
+    </row>
+    <row r="113" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="1"/>
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
@@ -3528,8 +3660,9 @@
       <c r="X113" s="1"/>
       <c r="Y113" s="1"/>
       <c r="Z113" s="1"/>
-    </row>
-    <row r="114" ht="15.75" customHeight="1">
+      <c r="AA113" s="1"/>
+    </row>
+    <row r="114" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
@@ -3556,8 +3689,9 @@
       <c r="X114" s="1"/>
       <c r="Y114" s="1"/>
       <c r="Z114" s="1"/>
-    </row>
-    <row r="115" ht="15.75" customHeight="1">
+      <c r="AA114" s="1"/>
+    </row>
+    <row r="115" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
@@ -3584,8 +3718,9 @@
       <c r="X115" s="1"/>
       <c r="Y115" s="1"/>
       <c r="Z115" s="1"/>
-    </row>
-    <row r="116" ht="15.75" customHeight="1">
+      <c r="AA115" s="1"/>
+    </row>
+    <row r="116" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
@@ -3612,8 +3747,9 @@
       <c r="X116" s="1"/>
       <c r="Y116" s="1"/>
       <c r="Z116" s="1"/>
-    </row>
-    <row r="117" ht="15.75" customHeight="1">
+      <c r="AA116" s="1"/>
+    </row>
+    <row r="117" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="1"/>
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
@@ -3640,8 +3776,9 @@
       <c r="X117" s="1"/>
       <c r="Y117" s="1"/>
       <c r="Z117" s="1"/>
-    </row>
-    <row r="118" ht="15.75" customHeight="1">
+      <c r="AA117" s="1"/>
+    </row>
+    <row r="118" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="1"/>
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
@@ -3668,8 +3805,9 @@
       <c r="X118" s="1"/>
       <c r="Y118" s="1"/>
       <c r="Z118" s="1"/>
-    </row>
-    <row r="119" ht="15.75" customHeight="1">
+      <c r="AA118" s="1"/>
+    </row>
+    <row r="119" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="1"/>
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
@@ -3696,8 +3834,9 @@
       <c r="X119" s="1"/>
       <c r="Y119" s="1"/>
       <c r="Z119" s="1"/>
-    </row>
-    <row r="120" ht="15.75" customHeight="1">
+      <c r="AA119" s="1"/>
+    </row>
+    <row r="120" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="1"/>
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
@@ -3724,8 +3863,9 @@
       <c r="X120" s="1"/>
       <c r="Y120" s="1"/>
       <c r="Z120" s="1"/>
-    </row>
-    <row r="121" ht="15.75" customHeight="1">
+      <c r="AA120" s="1"/>
+    </row>
+    <row r="121" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="1"/>
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
@@ -3752,8 +3892,9 @@
       <c r="X121" s="1"/>
       <c r="Y121" s="1"/>
       <c r="Z121" s="1"/>
-    </row>
-    <row r="122" ht="15.75" customHeight="1">
+      <c r="AA121" s="1"/>
+    </row>
+    <row r="122" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
@@ -3780,8 +3921,9 @@
       <c r="X122" s="1"/>
       <c r="Y122" s="1"/>
       <c r="Z122" s="1"/>
-    </row>
-    <row r="123" ht="15.75" customHeight="1">
+      <c r="AA122" s="1"/>
+    </row>
+    <row r="123" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="1"/>
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
@@ -3808,8 +3950,9 @@
       <c r="X123" s="1"/>
       <c r="Y123" s="1"/>
       <c r="Z123" s="1"/>
-    </row>
-    <row r="124" ht="15.75" customHeight="1">
+      <c r="AA123" s="1"/>
+    </row>
+    <row r="124" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1"/>
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
@@ -3836,8 +3979,9 @@
       <c r="X124" s="1"/>
       <c r="Y124" s="1"/>
       <c r="Z124" s="1"/>
-    </row>
-    <row r="125" ht="15.75" customHeight="1">
+      <c r="AA124" s="1"/>
+    </row>
+    <row r="125" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="1"/>
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
@@ -3864,8 +4008,9 @@
       <c r="X125" s="1"/>
       <c r="Y125" s="1"/>
       <c r="Z125" s="1"/>
-    </row>
-    <row r="126" ht="15.75" customHeight="1">
+      <c r="AA125" s="1"/>
+    </row>
+    <row r="126" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="1"/>
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
@@ -3892,8 +4037,9 @@
       <c r="X126" s="1"/>
       <c r="Y126" s="1"/>
       <c r="Z126" s="1"/>
-    </row>
-    <row r="127" ht="15.75" customHeight="1">
+      <c r="AA126" s="1"/>
+    </row>
+    <row r="127" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="1"/>
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
@@ -3920,8 +4066,9 @@
       <c r="X127" s="1"/>
       <c r="Y127" s="1"/>
       <c r="Z127" s="1"/>
-    </row>
-    <row r="128" ht="15.75" customHeight="1">
+      <c r="AA127" s="1"/>
+    </row>
+    <row r="128" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="1"/>
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
@@ -3948,8 +4095,9 @@
       <c r="X128" s="1"/>
       <c r="Y128" s="1"/>
       <c r="Z128" s="1"/>
-    </row>
-    <row r="129" ht="15.75" customHeight="1">
+      <c r="AA128" s="1"/>
+    </row>
+    <row r="129" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="1"/>
       <c r="B129" s="1"/>
       <c r="C129" s="1"/>
@@ -3976,8 +4124,9 @@
       <c r="X129" s="1"/>
       <c r="Y129" s="1"/>
       <c r="Z129" s="1"/>
-    </row>
-    <row r="130" ht="15.75" customHeight="1">
+      <c r="AA129" s="1"/>
+    </row>
+    <row r="130" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="1"/>
       <c r="B130" s="1"/>
       <c r="C130" s="1"/>
@@ -4004,8 +4153,9 @@
       <c r="X130" s="1"/>
       <c r="Y130" s="1"/>
       <c r="Z130" s="1"/>
-    </row>
-    <row r="131" ht="15.75" customHeight="1">
+      <c r="AA130" s="1"/>
+    </row>
+    <row r="131" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="1"/>
       <c r="B131" s="1"/>
       <c r="C131" s="1"/>
@@ -4032,8 +4182,9 @@
       <c r="X131" s="1"/>
       <c r="Y131" s="1"/>
       <c r="Z131" s="1"/>
-    </row>
-    <row r="132" ht="15.75" customHeight="1">
+      <c r="AA131" s="1"/>
+    </row>
+    <row r="132" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="1"/>
       <c r="B132" s="1"/>
       <c r="C132" s="1"/>
@@ -4060,8 +4211,9 @@
       <c r="X132" s="1"/>
       <c r="Y132" s="1"/>
       <c r="Z132" s="1"/>
-    </row>
-    <row r="133" ht="15.75" customHeight="1">
+      <c r="AA132" s="1"/>
+    </row>
+    <row r="133" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="1"/>
       <c r="B133" s="1"/>
       <c r="C133" s="1"/>
@@ -4088,8 +4240,9 @@
       <c r="X133" s="1"/>
       <c r="Y133" s="1"/>
       <c r="Z133" s="1"/>
-    </row>
-    <row r="134" ht="15.75" customHeight="1">
+      <c r="AA133" s="1"/>
+    </row>
+    <row r="134" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="1"/>
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
@@ -4116,8 +4269,9 @@
       <c r="X134" s="1"/>
       <c r="Y134" s="1"/>
       <c r="Z134" s="1"/>
-    </row>
-    <row r="135" ht="15.75" customHeight="1">
+      <c r="AA134" s="1"/>
+    </row>
+    <row r="135" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="1"/>
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
@@ -4144,8 +4298,9 @@
       <c r="X135" s="1"/>
       <c r="Y135" s="1"/>
       <c r="Z135" s="1"/>
-    </row>
-    <row r="136" ht="15.75" customHeight="1">
+      <c r="AA135" s="1"/>
+    </row>
+    <row r="136" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="1"/>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
@@ -4172,8 +4327,9 @@
       <c r="X136" s="1"/>
       <c r="Y136" s="1"/>
       <c r="Z136" s="1"/>
-    </row>
-    <row r="137" ht="15.75" customHeight="1">
+      <c r="AA136" s="1"/>
+    </row>
+    <row r="137" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="1"/>
       <c r="B137" s="1"/>
       <c r="C137" s="1"/>
@@ -4200,8 +4356,9 @@
       <c r="X137" s="1"/>
       <c r="Y137" s="1"/>
       <c r="Z137" s="1"/>
-    </row>
-    <row r="138" ht="15.75" customHeight="1">
+      <c r="AA137" s="1"/>
+    </row>
+    <row r="138" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="1"/>
       <c r="B138" s="1"/>
       <c r="C138" s="1"/>
@@ -4228,8 +4385,9 @@
       <c r="X138" s="1"/>
       <c r="Y138" s="1"/>
       <c r="Z138" s="1"/>
-    </row>
-    <row r="139" ht="15.75" customHeight="1">
+      <c r="AA138" s="1"/>
+    </row>
+    <row r="139" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="1"/>
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
@@ -4256,8 +4414,9 @@
       <c r="X139" s="1"/>
       <c r="Y139" s="1"/>
       <c r="Z139" s="1"/>
-    </row>
-    <row r="140" ht="15.75" customHeight="1">
+      <c r="AA139" s="1"/>
+    </row>
+    <row r="140" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="1"/>
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
@@ -4284,8 +4443,9 @@
       <c r="X140" s="1"/>
       <c r="Y140" s="1"/>
       <c r="Z140" s="1"/>
-    </row>
-    <row r="141" ht="15.75" customHeight="1">
+      <c r="AA140" s="1"/>
+    </row>
+    <row r="141" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="1"/>
       <c r="B141" s="1"/>
       <c r="C141" s="1"/>
@@ -4312,8 +4472,9 @@
       <c r="X141" s="1"/>
       <c r="Y141" s="1"/>
       <c r="Z141" s="1"/>
-    </row>
-    <row r="142" ht="15.75" customHeight="1">
+      <c r="AA141" s="1"/>
+    </row>
+    <row r="142" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
@@ -4340,8 +4501,9 @@
       <c r="X142" s="1"/>
       <c r="Y142" s="1"/>
       <c r="Z142" s="1"/>
-    </row>
-    <row r="143" ht="15.75" customHeight="1">
+      <c r="AA142" s="1"/>
+    </row>
+    <row r="143" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="1"/>
       <c r="B143" s="1"/>
       <c r="C143" s="1"/>
@@ -4368,8 +4530,9 @@
       <c r="X143" s="1"/>
       <c r="Y143" s="1"/>
       <c r="Z143" s="1"/>
-    </row>
-    <row r="144" ht="15.75" customHeight="1">
+      <c r="AA143" s="1"/>
+    </row>
+    <row r="144" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="1"/>
       <c r="B144" s="1"/>
       <c r="C144" s="1"/>
@@ -4396,8 +4559,9 @@
       <c r="X144" s="1"/>
       <c r="Y144" s="1"/>
       <c r="Z144" s="1"/>
-    </row>
-    <row r="145" ht="15.75" customHeight="1">
+      <c r="AA144" s="1"/>
+    </row>
+    <row r="145" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="1"/>
       <c r="B145" s="1"/>
       <c r="C145" s="1"/>
@@ -4424,8 +4588,9 @@
       <c r="X145" s="1"/>
       <c r="Y145" s="1"/>
       <c r="Z145" s="1"/>
-    </row>
-    <row r="146" ht="15.75" customHeight="1">
+      <c r="AA145" s="1"/>
+    </row>
+    <row r="146" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="1"/>
       <c r="B146" s="1"/>
       <c r="C146" s="1"/>
@@ -4452,8 +4617,9 @@
       <c r="X146" s="1"/>
       <c r="Y146" s="1"/>
       <c r="Z146" s="1"/>
-    </row>
-    <row r="147" ht="15.75" customHeight="1">
+      <c r="AA146" s="1"/>
+    </row>
+    <row r="147" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="1"/>
       <c r="B147" s="1"/>
       <c r="C147" s="1"/>
@@ -4480,8 +4646,9 @@
       <c r="X147" s="1"/>
       <c r="Y147" s="1"/>
       <c r="Z147" s="1"/>
-    </row>
-    <row r="148" ht="15.75" customHeight="1">
+      <c r="AA147" s="1"/>
+    </row>
+    <row r="148" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
@@ -4508,8 +4675,9 @@
       <c r="X148" s="1"/>
       <c r="Y148" s="1"/>
       <c r="Z148" s="1"/>
-    </row>
-    <row r="149" ht="15.75" customHeight="1">
+      <c r="AA148" s="1"/>
+    </row>
+    <row r="149" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="1"/>
       <c r="B149" s="1"/>
       <c r="C149" s="1"/>
@@ -4536,8 +4704,9 @@
       <c r="X149" s="1"/>
       <c r="Y149" s="1"/>
       <c r="Z149" s="1"/>
-    </row>
-    <row r="150" ht="15.75" customHeight="1">
+      <c r="AA149" s="1"/>
+    </row>
+    <row r="150" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="1"/>
       <c r="B150" s="1"/>
       <c r="C150" s="1"/>
@@ -4564,8 +4733,9 @@
       <c r="X150" s="1"/>
       <c r="Y150" s="1"/>
       <c r="Z150" s="1"/>
-    </row>
-    <row r="151" ht="15.75" customHeight="1">
+      <c r="AA150" s="1"/>
+    </row>
+    <row r="151" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="1"/>
       <c r="B151" s="1"/>
       <c r="C151" s="1"/>
@@ -4592,8 +4762,9 @@
       <c r="X151" s="1"/>
       <c r="Y151" s="1"/>
       <c r="Z151" s="1"/>
-    </row>
-    <row r="152" ht="15.75" customHeight="1">
+      <c r="AA151" s="1"/>
+    </row>
+    <row r="152" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="1"/>
       <c r="B152" s="1"/>
       <c r="C152" s="1"/>
@@ -4620,8 +4791,9 @@
       <c r="X152" s="1"/>
       <c r="Y152" s="1"/>
       <c r="Z152" s="1"/>
-    </row>
-    <row r="153" ht="15.75" customHeight="1">
+      <c r="AA152" s="1"/>
+    </row>
+    <row r="153" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="1"/>
       <c r="B153" s="1"/>
       <c r="C153" s="1"/>
@@ -4648,8 +4820,9 @@
       <c r="X153" s="1"/>
       <c r="Y153" s="1"/>
       <c r="Z153" s="1"/>
-    </row>
-    <row r="154" ht="15.75" customHeight="1">
+      <c r="AA153" s="1"/>
+    </row>
+    <row r="154" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
@@ -4676,8 +4849,9 @@
       <c r="X154" s="1"/>
       <c r="Y154" s="1"/>
       <c r="Z154" s="1"/>
-    </row>
-    <row r="155" ht="15.75" customHeight="1">
+      <c r="AA154" s="1"/>
+    </row>
+    <row r="155" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="1"/>
       <c r="B155" s="1"/>
       <c r="C155" s="1"/>
@@ -4704,8 +4878,9 @@
       <c r="X155" s="1"/>
       <c r="Y155" s="1"/>
       <c r="Z155" s="1"/>
-    </row>
-    <row r="156" ht="15.75" customHeight="1">
+      <c r="AA155" s="1"/>
+    </row>
+    <row r="156" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="1"/>
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
@@ -4732,8 +4907,9 @@
       <c r="X156" s="1"/>
       <c r="Y156" s="1"/>
       <c r="Z156" s="1"/>
-    </row>
-    <row r="157" ht="15.75" customHeight="1">
+      <c r="AA156" s="1"/>
+    </row>
+    <row r="157" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="1"/>
       <c r="B157" s="1"/>
       <c r="C157" s="1"/>
@@ -4760,8 +4936,9 @@
       <c r="X157" s="1"/>
       <c r="Y157" s="1"/>
       <c r="Z157" s="1"/>
-    </row>
-    <row r="158" ht="15.75" customHeight="1">
+      <c r="AA157" s="1"/>
+    </row>
+    <row r="158" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="1"/>
       <c r="B158" s="1"/>
       <c r="C158" s="1"/>
@@ -4788,8 +4965,9 @@
       <c r="X158" s="1"/>
       <c r="Y158" s="1"/>
       <c r="Z158" s="1"/>
-    </row>
-    <row r="159" ht="15.75" customHeight="1">
+      <c r="AA158" s="1"/>
+    </row>
+    <row r="159" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="1"/>
       <c r="B159" s="1"/>
       <c r="C159" s="1"/>
@@ -4816,8 +4994,9 @@
       <c r="X159" s="1"/>
       <c r="Y159" s="1"/>
       <c r="Z159" s="1"/>
-    </row>
-    <row r="160" ht="15.75" customHeight="1">
+      <c r="AA159" s="1"/>
+    </row>
+    <row r="160" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="1"/>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
@@ -4844,8 +5023,9 @@
       <c r="X160" s="1"/>
       <c r="Y160" s="1"/>
       <c r="Z160" s="1"/>
-    </row>
-    <row r="161" ht="15.75" customHeight="1">
+      <c r="AA160" s="1"/>
+    </row>
+    <row r="161" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="1"/>
       <c r="B161" s="1"/>
       <c r="C161" s="1"/>
@@ -4872,8 +5052,9 @@
       <c r="X161" s="1"/>
       <c r="Y161" s="1"/>
       <c r="Z161" s="1"/>
-    </row>
-    <row r="162" ht="15.75" customHeight="1">
+      <c r="AA161" s="1"/>
+    </row>
+    <row r="162" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="1"/>
       <c r="B162" s="1"/>
       <c r="C162" s="1"/>
@@ -4900,8 +5081,9 @@
       <c r="X162" s="1"/>
       <c r="Y162" s="1"/>
       <c r="Z162" s="1"/>
-    </row>
-    <row r="163" ht="15.75" customHeight="1">
+      <c r="AA162" s="1"/>
+    </row>
+    <row r="163" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="1"/>
       <c r="B163" s="1"/>
       <c r="C163" s="1"/>
@@ -4928,8 +5110,9 @@
       <c r="X163" s="1"/>
       <c r="Y163" s="1"/>
       <c r="Z163" s="1"/>
-    </row>
-    <row r="164" ht="15.75" customHeight="1">
+      <c r="AA163" s="1"/>
+    </row>
+    <row r="164" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="1"/>
       <c r="B164" s="1"/>
       <c r="C164" s="1"/>
@@ -4956,8 +5139,9 @@
       <c r="X164" s="1"/>
       <c r="Y164" s="1"/>
       <c r="Z164" s="1"/>
-    </row>
-    <row r="165" ht="15.75" customHeight="1">
+      <c r="AA164" s="1"/>
+    </row>
+    <row r="165" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="1"/>
       <c r="B165" s="1"/>
       <c r="C165" s="1"/>
@@ -4984,8 +5168,9 @@
       <c r="X165" s="1"/>
       <c r="Y165" s="1"/>
       <c r="Z165" s="1"/>
-    </row>
-    <row r="166" ht="15.75" customHeight="1">
+      <c r="AA165" s="1"/>
+    </row>
+    <row r="166" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="1"/>
       <c r="B166" s="1"/>
       <c r="C166" s="1"/>
@@ -5012,8 +5197,9 @@
       <c r="X166" s="1"/>
       <c r="Y166" s="1"/>
       <c r="Z166" s="1"/>
-    </row>
-    <row r="167" ht="15.75" customHeight="1">
+      <c r="AA166" s="1"/>
+    </row>
+    <row r="167" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="1"/>
       <c r="B167" s="1"/>
       <c r="C167" s="1"/>
@@ -5040,8 +5226,9 @@
       <c r="X167" s="1"/>
       <c r="Y167" s="1"/>
       <c r="Z167" s="1"/>
-    </row>
-    <row r="168" ht="15.75" customHeight="1">
+      <c r="AA167" s="1"/>
+    </row>
+    <row r="168" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="1"/>
       <c r="B168" s="1"/>
       <c r="C168" s="1"/>
@@ -5068,8 +5255,9 @@
       <c r="X168" s="1"/>
       <c r="Y168" s="1"/>
       <c r="Z168" s="1"/>
-    </row>
-    <row r="169" ht="15.75" customHeight="1">
+      <c r="AA168" s="1"/>
+    </row>
+    <row r="169" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="1"/>
       <c r="B169" s="1"/>
       <c r="C169" s="1"/>
@@ -5096,8 +5284,9 @@
       <c r="X169" s="1"/>
       <c r="Y169" s="1"/>
       <c r="Z169" s="1"/>
-    </row>
-    <row r="170" ht="15.75" customHeight="1">
+      <c r="AA169" s="1"/>
+    </row>
+    <row r="170" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="1"/>
       <c r="B170" s="1"/>
       <c r="C170" s="1"/>
@@ -5124,8 +5313,9 @@
       <c r="X170" s="1"/>
       <c r="Y170" s="1"/>
       <c r="Z170" s="1"/>
-    </row>
-    <row r="171" ht="15.75" customHeight="1">
+      <c r="AA170" s="1"/>
+    </row>
+    <row r="171" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="1"/>
       <c r="B171" s="1"/>
       <c r="C171" s="1"/>
@@ -5152,8 +5342,9 @@
       <c r="X171" s="1"/>
       <c r="Y171" s="1"/>
       <c r="Z171" s="1"/>
-    </row>
-    <row r="172" ht="15.75" customHeight="1">
+      <c r="AA171" s="1"/>
+    </row>
+    <row r="172" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="1"/>
       <c r="B172" s="1"/>
       <c r="C172" s="1"/>
@@ -5180,8 +5371,9 @@
       <c r="X172" s="1"/>
       <c r="Y172" s="1"/>
       <c r="Z172" s="1"/>
-    </row>
-    <row r="173" ht="15.75" customHeight="1">
+      <c r="AA172" s="1"/>
+    </row>
+    <row r="173" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="1"/>
       <c r="B173" s="1"/>
       <c r="C173" s="1"/>
@@ -5208,8 +5400,9 @@
       <c r="X173" s="1"/>
       <c r="Y173" s="1"/>
       <c r="Z173" s="1"/>
-    </row>
-    <row r="174" ht="15.75" customHeight="1">
+      <c r="AA173" s="1"/>
+    </row>
+    <row r="174" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="1"/>
       <c r="B174" s="1"/>
       <c r="C174" s="1"/>
@@ -5236,8 +5429,9 @@
       <c r="X174" s="1"/>
       <c r="Y174" s="1"/>
       <c r="Z174" s="1"/>
-    </row>
-    <row r="175" ht="15.75" customHeight="1">
+      <c r="AA174" s="1"/>
+    </row>
+    <row r="175" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="1"/>
       <c r="B175" s="1"/>
       <c r="C175" s="1"/>
@@ -5264,8 +5458,9 @@
       <c r="X175" s="1"/>
       <c r="Y175" s="1"/>
       <c r="Z175" s="1"/>
-    </row>
-    <row r="176" ht="15.75" customHeight="1">
+      <c r="AA175" s="1"/>
+    </row>
+    <row r="176" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="1"/>
       <c r="B176" s="1"/>
       <c r="C176" s="1"/>
@@ -5292,8 +5487,9 @@
       <c r="X176" s="1"/>
       <c r="Y176" s="1"/>
       <c r="Z176" s="1"/>
-    </row>
-    <row r="177" ht="15.75" customHeight="1">
+      <c r="AA176" s="1"/>
+    </row>
+    <row r="177" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="1"/>
       <c r="B177" s="1"/>
       <c r="C177" s="1"/>
@@ -5320,8 +5516,9 @@
       <c r="X177" s="1"/>
       <c r="Y177" s="1"/>
       <c r="Z177" s="1"/>
-    </row>
-    <row r="178" ht="15.75" customHeight="1">
+      <c r="AA177" s="1"/>
+    </row>
+    <row r="178" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="1"/>
       <c r="B178" s="1"/>
       <c r="C178" s="1"/>
@@ -5348,8 +5545,9 @@
       <c r="X178" s="1"/>
       <c r="Y178" s="1"/>
       <c r="Z178" s="1"/>
-    </row>
-    <row r="179" ht="15.75" customHeight="1">
+      <c r="AA178" s="1"/>
+    </row>
+    <row r="179" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="1"/>
       <c r="B179" s="1"/>
       <c r="C179" s="1"/>
@@ -5376,8 +5574,9 @@
       <c r="X179" s="1"/>
       <c r="Y179" s="1"/>
       <c r="Z179" s="1"/>
-    </row>
-    <row r="180" ht="15.75" customHeight="1">
+      <c r="AA179" s="1"/>
+    </row>
+    <row r="180" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="1"/>
       <c r="B180" s="1"/>
       <c r="C180" s="1"/>
@@ -5404,8 +5603,9 @@
       <c r="X180" s="1"/>
       <c r="Y180" s="1"/>
       <c r="Z180" s="1"/>
-    </row>
-    <row r="181" ht="15.75" customHeight="1">
+      <c r="AA180" s="1"/>
+    </row>
+    <row r="181" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="1"/>
       <c r="B181" s="1"/>
       <c r="C181" s="1"/>
@@ -5432,8 +5632,9 @@
       <c r="X181" s="1"/>
       <c r="Y181" s="1"/>
       <c r="Z181" s="1"/>
-    </row>
-    <row r="182" ht="15.75" customHeight="1">
+      <c r="AA181" s="1"/>
+    </row>
+    <row r="182" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="1"/>
       <c r="B182" s="1"/>
       <c r="C182" s="1"/>
@@ -5460,8 +5661,9 @@
       <c r="X182" s="1"/>
       <c r="Y182" s="1"/>
       <c r="Z182" s="1"/>
-    </row>
-    <row r="183" ht="15.75" customHeight="1">
+      <c r="AA182" s="1"/>
+    </row>
+    <row r="183" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="1"/>
       <c r="B183" s="1"/>
       <c r="C183" s="1"/>
@@ -5488,8 +5690,9 @@
       <c r="X183" s="1"/>
       <c r="Y183" s="1"/>
       <c r="Z183" s="1"/>
-    </row>
-    <row r="184" ht="15.75" customHeight="1">
+      <c r="AA183" s="1"/>
+    </row>
+    <row r="184" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="1"/>
       <c r="B184" s="1"/>
       <c r="C184" s="1"/>
@@ -5516,8 +5719,9 @@
       <c r="X184" s="1"/>
       <c r="Y184" s="1"/>
       <c r="Z184" s="1"/>
-    </row>
-    <row r="185" ht="15.75" customHeight="1">
+      <c r="AA184" s="1"/>
+    </row>
+    <row r="185" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="1"/>
       <c r="B185" s="1"/>
       <c r="C185" s="1"/>
@@ -5544,8 +5748,9 @@
       <c r="X185" s="1"/>
       <c r="Y185" s="1"/>
       <c r="Z185" s="1"/>
-    </row>
-    <row r="186" ht="15.75" customHeight="1">
+      <c r="AA185" s="1"/>
+    </row>
+    <row r="186" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="1"/>
       <c r="B186" s="1"/>
       <c r="C186" s="1"/>
@@ -5572,8 +5777,9 @@
       <c r="X186" s="1"/>
       <c r="Y186" s="1"/>
       <c r="Z186" s="1"/>
-    </row>
-    <row r="187" ht="15.75" customHeight="1">
+      <c r="AA186" s="1"/>
+    </row>
+    <row r="187" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="1"/>
       <c r="B187" s="1"/>
       <c r="C187" s="1"/>
@@ -5600,8 +5806,9 @@
       <c r="X187" s="1"/>
       <c r="Y187" s="1"/>
       <c r="Z187" s="1"/>
-    </row>
-    <row r="188" ht="15.75" customHeight="1">
+      <c r="AA187" s="1"/>
+    </row>
+    <row r="188" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="1"/>
       <c r="B188" s="1"/>
       <c r="C188" s="1"/>
@@ -5628,8 +5835,9 @@
       <c r="X188" s="1"/>
       <c r="Y188" s="1"/>
       <c r="Z188" s="1"/>
-    </row>
-    <row r="189" ht="15.75" customHeight="1">
+      <c r="AA188" s="1"/>
+    </row>
+    <row r="189" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="1"/>
       <c r="B189" s="1"/>
       <c r="C189" s="1"/>
@@ -5656,8 +5864,9 @@
       <c r="X189" s="1"/>
       <c r="Y189" s="1"/>
       <c r="Z189" s="1"/>
-    </row>
-    <row r="190" ht="15.75" customHeight="1">
+      <c r="AA189" s="1"/>
+    </row>
+    <row r="190" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="1"/>
       <c r="B190" s="1"/>
       <c r="C190" s="1"/>
@@ -5684,8 +5893,9 @@
       <c r="X190" s="1"/>
       <c r="Y190" s="1"/>
       <c r="Z190" s="1"/>
-    </row>
-    <row r="191" ht="15.75" customHeight="1">
+      <c r="AA190" s="1"/>
+    </row>
+    <row r="191" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="1"/>
       <c r="B191" s="1"/>
       <c r="C191" s="1"/>
@@ -5712,8 +5922,9 @@
       <c r="X191" s="1"/>
       <c r="Y191" s="1"/>
       <c r="Z191" s="1"/>
-    </row>
-    <row r="192" ht="15.75" customHeight="1">
+      <c r="AA191" s="1"/>
+    </row>
+    <row r="192" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="1"/>
       <c r="B192" s="1"/>
       <c r="C192" s="1"/>
@@ -5740,8 +5951,9 @@
       <c r="X192" s="1"/>
       <c r="Y192" s="1"/>
       <c r="Z192" s="1"/>
-    </row>
-    <row r="193" ht="15.75" customHeight="1">
+      <c r="AA192" s="1"/>
+    </row>
+    <row r="193" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="1"/>
       <c r="B193" s="1"/>
       <c r="C193" s="1"/>
@@ -5768,8 +5980,9 @@
       <c r="X193" s="1"/>
       <c r="Y193" s="1"/>
       <c r="Z193" s="1"/>
-    </row>
-    <row r="194" ht="15.75" customHeight="1">
+      <c r="AA193" s="1"/>
+    </row>
+    <row r="194" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="1"/>
       <c r="B194" s="1"/>
       <c r="C194" s="1"/>
@@ -5796,8 +6009,9 @@
       <c r="X194" s="1"/>
       <c r="Y194" s="1"/>
       <c r="Z194" s="1"/>
-    </row>
-    <row r="195" ht="15.75" customHeight="1">
+      <c r="AA194" s="1"/>
+    </row>
+    <row r="195" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="1"/>
       <c r="B195" s="1"/>
       <c r="C195" s="1"/>
@@ -5824,8 +6038,9 @@
       <c r="X195" s="1"/>
       <c r="Y195" s="1"/>
       <c r="Z195" s="1"/>
-    </row>
-    <row r="196" ht="15.75" customHeight="1">
+      <c r="AA195" s="1"/>
+    </row>
+    <row r="196" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="1"/>
       <c r="B196" s="1"/>
       <c r="C196" s="1"/>
@@ -5852,8 +6067,9 @@
       <c r="X196" s="1"/>
       <c r="Y196" s="1"/>
       <c r="Z196" s="1"/>
-    </row>
-    <row r="197" ht="15.75" customHeight="1">
+      <c r="AA196" s="1"/>
+    </row>
+    <row r="197" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="1"/>
       <c r="B197" s="1"/>
       <c r="C197" s="1"/>
@@ -5880,8 +6096,9 @@
       <c r="X197" s="1"/>
       <c r="Y197" s="1"/>
       <c r="Z197" s="1"/>
-    </row>
-    <row r="198" ht="15.75" customHeight="1">
+      <c r="AA197" s="1"/>
+    </row>
+    <row r="198" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="1"/>
       <c r="B198" s="1"/>
       <c r="C198" s="1"/>
@@ -5908,8 +6125,9 @@
       <c r="X198" s="1"/>
       <c r="Y198" s="1"/>
       <c r="Z198" s="1"/>
-    </row>
-    <row r="199" ht="15.75" customHeight="1">
+      <c r="AA198" s="1"/>
+    </row>
+    <row r="199" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="1"/>
       <c r="B199" s="1"/>
       <c r="C199" s="1"/>
@@ -5936,8 +6154,9 @@
       <c r="X199" s="1"/>
       <c r="Y199" s="1"/>
       <c r="Z199" s="1"/>
-    </row>
-    <row r="200" ht="15.75" customHeight="1">
+      <c r="AA199" s="1"/>
+    </row>
+    <row r="200" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="1"/>
       <c r="B200" s="1"/>
       <c r="C200" s="1"/>
@@ -5964,8 +6183,9 @@
       <c r="X200" s="1"/>
       <c r="Y200" s="1"/>
       <c r="Z200" s="1"/>
-    </row>
-    <row r="201" ht="15.75" customHeight="1">
+      <c r="AA200" s="1"/>
+    </row>
+    <row r="201" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="1"/>
       <c r="B201" s="1"/>
       <c r="C201" s="1"/>
@@ -5992,8 +6212,9 @@
       <c r="X201" s="1"/>
       <c r="Y201" s="1"/>
       <c r="Z201" s="1"/>
-    </row>
-    <row r="202" ht="15.75" customHeight="1">
+      <c r="AA201" s="1"/>
+    </row>
+    <row r="202" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A202" s="1"/>
       <c r="B202" s="1"/>
       <c r="C202" s="1"/>
@@ -6020,8 +6241,9 @@
       <c r="X202" s="1"/>
       <c r="Y202" s="1"/>
       <c r="Z202" s="1"/>
-    </row>
-    <row r="203" ht="15.75" customHeight="1">
+      <c r="AA202" s="1"/>
+    </row>
+    <row r="203" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A203" s="1"/>
       <c r="B203" s="1"/>
       <c r="C203" s="1"/>
@@ -6048,8 +6270,9 @@
       <c r="X203" s="1"/>
       <c r="Y203" s="1"/>
       <c r="Z203" s="1"/>
-    </row>
-    <row r="204" ht="15.75" customHeight="1">
+      <c r="AA203" s="1"/>
+    </row>
+    <row r="204" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="1"/>
       <c r="B204" s="1"/>
       <c r="C204" s="1"/>
@@ -6076,8 +6299,9 @@
       <c r="X204" s="1"/>
       <c r="Y204" s="1"/>
       <c r="Z204" s="1"/>
-    </row>
-    <row r="205" ht="15.75" customHeight="1">
+      <c r="AA204" s="1"/>
+    </row>
+    <row r="205" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="1"/>
       <c r="B205" s="1"/>
       <c r="C205" s="1"/>
@@ -6104,8 +6328,9 @@
       <c r="X205" s="1"/>
       <c r="Y205" s="1"/>
       <c r="Z205" s="1"/>
-    </row>
-    <row r="206" ht="15.75" customHeight="1">
+      <c r="AA205" s="1"/>
+    </row>
+    <row r="206" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="1"/>
       <c r="B206" s="1"/>
       <c r="C206" s="1"/>
@@ -6132,8 +6357,9 @@
       <c r="X206" s="1"/>
       <c r="Y206" s="1"/>
       <c r="Z206" s="1"/>
-    </row>
-    <row r="207" ht="15.75" customHeight="1">
+      <c r="AA206" s="1"/>
+    </row>
+    <row r="207" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="1"/>
       <c r="B207" s="1"/>
       <c r="C207" s="1"/>
@@ -6160,8 +6386,9 @@
       <c r="X207" s="1"/>
       <c r="Y207" s="1"/>
       <c r="Z207" s="1"/>
-    </row>
-    <row r="208" ht="15.75" customHeight="1">
+      <c r="AA207" s="1"/>
+    </row>
+    <row r="208" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="1"/>
       <c r="B208" s="1"/>
       <c r="C208" s="1"/>
@@ -6188,8 +6415,9 @@
       <c r="X208" s="1"/>
       <c r="Y208" s="1"/>
       <c r="Z208" s="1"/>
-    </row>
-    <row r="209" ht="15.75" customHeight="1">
+      <c r="AA208" s="1"/>
+    </row>
+    <row r="209" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A209" s="1"/>
       <c r="B209" s="1"/>
       <c r="C209" s="1"/>
@@ -6216,8 +6444,9 @@
       <c r="X209" s="1"/>
       <c r="Y209" s="1"/>
       <c r="Z209" s="1"/>
-    </row>
-    <row r="210" ht="15.75" customHeight="1">
+      <c r="AA209" s="1"/>
+    </row>
+    <row r="210" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A210" s="1"/>
       <c r="B210" s="1"/>
       <c r="C210" s="1"/>
@@ -6244,8 +6473,9 @@
       <c r="X210" s="1"/>
       <c r="Y210" s="1"/>
       <c r="Z210" s="1"/>
-    </row>
-    <row r="211" ht="15.75" customHeight="1">
+      <c r="AA210" s="1"/>
+    </row>
+    <row r="211" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A211" s="1"/>
       <c r="B211" s="1"/>
       <c r="C211" s="1"/>
@@ -6272,8 +6502,9 @@
       <c r="X211" s="1"/>
       <c r="Y211" s="1"/>
       <c r="Z211" s="1"/>
-    </row>
-    <row r="212" ht="15.75" customHeight="1">
+      <c r="AA211" s="1"/>
+    </row>
+    <row r="212" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A212" s="1"/>
       <c r="B212" s="1"/>
       <c r="C212" s="1"/>
@@ -6300,8 +6531,9 @@
       <c r="X212" s="1"/>
       <c r="Y212" s="1"/>
       <c r="Z212" s="1"/>
-    </row>
-    <row r="213" ht="15.75" customHeight="1">
+      <c r="AA212" s="1"/>
+    </row>
+    <row r="213" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A213" s="1"/>
       <c r="B213" s="1"/>
       <c r="C213" s="1"/>
@@ -6328,8 +6560,9 @@
       <c r="X213" s="1"/>
       <c r="Y213" s="1"/>
       <c r="Z213" s="1"/>
-    </row>
-    <row r="214" ht="15.75" customHeight="1">
+      <c r="AA213" s="1"/>
+    </row>
+    <row r="214" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="1"/>
       <c r="B214" s="1"/>
       <c r="C214" s="1"/>
@@ -6356,8 +6589,9 @@
       <c r="X214" s="1"/>
       <c r="Y214" s="1"/>
       <c r="Z214" s="1"/>
-    </row>
-    <row r="215" ht="15.75" customHeight="1">
+      <c r="AA214" s="1"/>
+    </row>
+    <row r="215" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A215" s="1"/>
       <c r="B215" s="1"/>
       <c r="C215" s="1"/>
@@ -6384,8 +6618,9 @@
       <c r="X215" s="1"/>
       <c r="Y215" s="1"/>
       <c r="Z215" s="1"/>
-    </row>
-    <row r="216" ht="15.75" customHeight="1">
+      <c r="AA215" s="1"/>
+    </row>
+    <row r="216" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A216" s="1"/>
       <c r="B216" s="1"/>
       <c r="C216" s="1"/>
@@ -6412,8 +6647,9 @@
       <c r="X216" s="1"/>
       <c r="Y216" s="1"/>
       <c r="Z216" s="1"/>
-    </row>
-    <row r="217" ht="15.75" customHeight="1">
+      <c r="AA216" s="1"/>
+    </row>
+    <row r="217" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A217" s="1"/>
       <c r="B217" s="1"/>
       <c r="C217" s="1"/>
@@ -6440,8 +6676,9 @@
       <c r="X217" s="1"/>
       <c r="Y217" s="1"/>
       <c r="Z217" s="1"/>
-    </row>
-    <row r="218" ht="15.75" customHeight="1">
+      <c r="AA217" s="1"/>
+    </row>
+    <row r="218" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="1"/>
       <c r="B218" s="1"/>
       <c r="C218" s="1"/>
@@ -6468,8 +6705,9 @@
       <c r="X218" s="1"/>
       <c r="Y218" s="1"/>
       <c r="Z218" s="1"/>
-    </row>
-    <row r="219" ht="15.75" customHeight="1">
+      <c r="AA218" s="1"/>
+    </row>
+    <row r="219" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A219" s="1"/>
       <c r="B219" s="1"/>
       <c r="C219" s="1"/>
@@ -6496,8 +6734,9 @@
       <c r="X219" s="1"/>
       <c r="Y219" s="1"/>
       <c r="Z219" s="1"/>
-    </row>
-    <row r="220" ht="15.75" customHeight="1">
+      <c r="AA219" s="1"/>
+    </row>
+    <row r="220" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A220" s="1"/>
       <c r="B220" s="1"/>
       <c r="C220" s="1"/>
@@ -6524,791 +6763,790 @@
       <c r="X220" s="1"/>
       <c r="Y220" s="1"/>
       <c r="Z220" s="1"/>
-    </row>
-    <row r="221" ht="15.75" customHeight="1"/>
-    <row r="222" ht="15.75" customHeight="1"/>
-    <row r="223" ht="15.75" customHeight="1"/>
-    <row r="224" ht="15.75" customHeight="1"/>
-    <row r="225" ht="15.75" customHeight="1"/>
-    <row r="226" ht="15.75" customHeight="1"/>
-    <row r="227" ht="15.75" customHeight="1"/>
-    <row r="228" ht="15.75" customHeight="1"/>
-    <row r="229" ht="15.75" customHeight="1"/>
-    <row r="230" ht="15.75" customHeight="1"/>
-    <row r="231" ht="15.75" customHeight="1"/>
-    <row r="232" ht="15.75" customHeight="1"/>
-    <row r="233" ht="15.75" customHeight="1"/>
-    <row r="234" ht="15.75" customHeight="1"/>
-    <row r="235" ht="15.75" customHeight="1"/>
-    <row r="236" ht="15.75" customHeight="1"/>
-    <row r="237" ht="15.75" customHeight="1"/>
-    <row r="238" ht="15.75" customHeight="1"/>
-    <row r="239" ht="15.75" customHeight="1"/>
-    <row r="240" ht="15.75" customHeight="1"/>
-    <row r="241" ht="15.75" customHeight="1"/>
-    <row r="242" ht="15.75" customHeight="1"/>
-    <row r="243" ht="15.75" customHeight="1"/>
-    <row r="244" ht="15.75" customHeight="1"/>
-    <row r="245" ht="15.75" customHeight="1"/>
-    <row r="246" ht="15.75" customHeight="1"/>
-    <row r="247" ht="15.75" customHeight="1"/>
-    <row r="248" ht="15.75" customHeight="1"/>
-    <row r="249" ht="15.75" customHeight="1"/>
-    <row r="250" ht="15.75" customHeight="1"/>
-    <row r="251" ht="15.75" customHeight="1"/>
-    <row r="252" ht="15.75" customHeight="1"/>
-    <row r="253" ht="15.75" customHeight="1"/>
-    <row r="254" ht="15.75" customHeight="1"/>
-    <row r="255" ht="15.75" customHeight="1"/>
-    <row r="256" ht="15.75" customHeight="1"/>
-    <row r="257" ht="15.75" customHeight="1"/>
-    <row r="258" ht="15.75" customHeight="1"/>
-    <row r="259" ht="15.75" customHeight="1"/>
-    <row r="260" ht="15.75" customHeight="1"/>
-    <row r="261" ht="15.75" customHeight="1"/>
-    <row r="262" ht="15.75" customHeight="1"/>
-    <row r="263" ht="15.75" customHeight="1"/>
-    <row r="264" ht="15.75" customHeight="1"/>
-    <row r="265" ht="15.75" customHeight="1"/>
-    <row r="266" ht="15.75" customHeight="1"/>
-    <row r="267" ht="15.75" customHeight="1"/>
-    <row r="268" ht="15.75" customHeight="1"/>
-    <row r="269" ht="15.75" customHeight="1"/>
-    <row r="270" ht="15.75" customHeight="1"/>
-    <row r="271" ht="15.75" customHeight="1"/>
-    <row r="272" ht="15.75" customHeight="1"/>
-    <row r="273" ht="15.75" customHeight="1"/>
-    <row r="274" ht="15.75" customHeight="1"/>
-    <row r="275" ht="15.75" customHeight="1"/>
-    <row r="276" ht="15.75" customHeight="1"/>
-    <row r="277" ht="15.75" customHeight="1"/>
-    <row r="278" ht="15.75" customHeight="1"/>
-    <row r="279" ht="15.75" customHeight="1"/>
-    <row r="280" ht="15.75" customHeight="1"/>
-    <row r="281" ht="15.75" customHeight="1"/>
-    <row r="282" ht="15.75" customHeight="1"/>
-    <row r="283" ht="15.75" customHeight="1"/>
-    <row r="284" ht="15.75" customHeight="1"/>
-    <row r="285" ht="15.75" customHeight="1"/>
-    <row r="286" ht="15.75" customHeight="1"/>
-    <row r="287" ht="15.75" customHeight="1"/>
-    <row r="288" ht="15.75" customHeight="1"/>
-    <row r="289" ht="15.75" customHeight="1"/>
-    <row r="290" ht="15.75" customHeight="1"/>
-    <row r="291" ht="15.75" customHeight="1"/>
-    <row r="292" ht="15.75" customHeight="1"/>
-    <row r="293" ht="15.75" customHeight="1"/>
-    <row r="294" ht="15.75" customHeight="1"/>
-    <row r="295" ht="15.75" customHeight="1"/>
-    <row r="296" ht="15.75" customHeight="1"/>
-    <row r="297" ht="15.75" customHeight="1"/>
-    <row r="298" ht="15.75" customHeight="1"/>
-    <row r="299" ht="15.75" customHeight="1"/>
-    <row r="300" ht="15.75" customHeight="1"/>
-    <row r="301" ht="15.75" customHeight="1"/>
-    <row r="302" ht="15.75" customHeight="1"/>
-    <row r="303" ht="15.75" customHeight="1"/>
-    <row r="304" ht="15.75" customHeight="1"/>
-    <row r="305" ht="15.75" customHeight="1"/>
-    <row r="306" ht="15.75" customHeight="1"/>
-    <row r="307" ht="15.75" customHeight="1"/>
-    <row r="308" ht="15.75" customHeight="1"/>
-    <row r="309" ht="15.75" customHeight="1"/>
-    <row r="310" ht="15.75" customHeight="1"/>
-    <row r="311" ht="15.75" customHeight="1"/>
-    <row r="312" ht="15.75" customHeight="1"/>
-    <row r="313" ht="15.75" customHeight="1"/>
-    <row r="314" ht="15.75" customHeight="1"/>
-    <row r="315" ht="15.75" customHeight="1"/>
-    <row r="316" ht="15.75" customHeight="1"/>
-    <row r="317" ht="15.75" customHeight="1"/>
-    <row r="318" ht="15.75" customHeight="1"/>
-    <row r="319" ht="15.75" customHeight="1"/>
-    <row r="320" ht="15.75" customHeight="1"/>
-    <row r="321" ht="15.75" customHeight="1"/>
-    <row r="322" ht="15.75" customHeight="1"/>
-    <row r="323" ht="15.75" customHeight="1"/>
-    <row r="324" ht="15.75" customHeight="1"/>
-    <row r="325" ht="15.75" customHeight="1"/>
-    <row r="326" ht="15.75" customHeight="1"/>
-    <row r="327" ht="15.75" customHeight="1"/>
-    <row r="328" ht="15.75" customHeight="1"/>
-    <row r="329" ht="15.75" customHeight="1"/>
-    <row r="330" ht="15.75" customHeight="1"/>
-    <row r="331" ht="15.75" customHeight="1"/>
-    <row r="332" ht="15.75" customHeight="1"/>
-    <row r="333" ht="15.75" customHeight="1"/>
-    <row r="334" ht="15.75" customHeight="1"/>
-    <row r="335" ht="15.75" customHeight="1"/>
-    <row r="336" ht="15.75" customHeight="1"/>
-    <row r="337" ht="15.75" customHeight="1"/>
-    <row r="338" ht="15.75" customHeight="1"/>
-    <row r="339" ht="15.75" customHeight="1"/>
-    <row r="340" ht="15.75" customHeight="1"/>
-    <row r="341" ht="15.75" customHeight="1"/>
-    <row r="342" ht="15.75" customHeight="1"/>
-    <row r="343" ht="15.75" customHeight="1"/>
-    <row r="344" ht="15.75" customHeight="1"/>
-    <row r="345" ht="15.75" customHeight="1"/>
-    <row r="346" ht="15.75" customHeight="1"/>
-    <row r="347" ht="15.75" customHeight="1"/>
-    <row r="348" ht="15.75" customHeight="1"/>
-    <row r="349" ht="15.75" customHeight="1"/>
-    <row r="350" ht="15.75" customHeight="1"/>
-    <row r="351" ht="15.75" customHeight="1"/>
-    <row r="352" ht="15.75" customHeight="1"/>
-    <row r="353" ht="15.75" customHeight="1"/>
-    <row r="354" ht="15.75" customHeight="1"/>
-    <row r="355" ht="15.75" customHeight="1"/>
-    <row r="356" ht="15.75" customHeight="1"/>
-    <row r="357" ht="15.75" customHeight="1"/>
-    <row r="358" ht="15.75" customHeight="1"/>
-    <row r="359" ht="15.75" customHeight="1"/>
-    <row r="360" ht="15.75" customHeight="1"/>
-    <row r="361" ht="15.75" customHeight="1"/>
-    <row r="362" ht="15.75" customHeight="1"/>
-    <row r="363" ht="15.75" customHeight="1"/>
-    <row r="364" ht="15.75" customHeight="1"/>
-    <row r="365" ht="15.75" customHeight="1"/>
-    <row r="366" ht="15.75" customHeight="1"/>
-    <row r="367" ht="15.75" customHeight="1"/>
-    <row r="368" ht="15.75" customHeight="1"/>
-    <row r="369" ht="15.75" customHeight="1"/>
-    <row r="370" ht="15.75" customHeight="1"/>
-    <row r="371" ht="15.75" customHeight="1"/>
-    <row r="372" ht="15.75" customHeight="1"/>
-    <row r="373" ht="15.75" customHeight="1"/>
-    <row r="374" ht="15.75" customHeight="1"/>
-    <row r="375" ht="15.75" customHeight="1"/>
-    <row r="376" ht="15.75" customHeight="1"/>
-    <row r="377" ht="15.75" customHeight="1"/>
-    <row r="378" ht="15.75" customHeight="1"/>
-    <row r="379" ht="15.75" customHeight="1"/>
-    <row r="380" ht="15.75" customHeight="1"/>
-    <row r="381" ht="15.75" customHeight="1"/>
-    <row r="382" ht="15.75" customHeight="1"/>
-    <row r="383" ht="15.75" customHeight="1"/>
-    <row r="384" ht="15.75" customHeight="1"/>
-    <row r="385" ht="15.75" customHeight="1"/>
-    <row r="386" ht="15.75" customHeight="1"/>
-    <row r="387" ht="15.75" customHeight="1"/>
-    <row r="388" ht="15.75" customHeight="1"/>
-    <row r="389" ht="15.75" customHeight="1"/>
-    <row r="390" ht="15.75" customHeight="1"/>
-    <row r="391" ht="15.75" customHeight="1"/>
-    <row r="392" ht="15.75" customHeight="1"/>
-    <row r="393" ht="15.75" customHeight="1"/>
-    <row r="394" ht="15.75" customHeight="1"/>
-    <row r="395" ht="15.75" customHeight="1"/>
-    <row r="396" ht="15.75" customHeight="1"/>
-    <row r="397" ht="15.75" customHeight="1"/>
-    <row r="398" ht="15.75" customHeight="1"/>
-    <row r="399" ht="15.75" customHeight="1"/>
-    <row r="400" ht="15.75" customHeight="1"/>
-    <row r="401" ht="15.75" customHeight="1"/>
-    <row r="402" ht="15.75" customHeight="1"/>
-    <row r="403" ht="15.75" customHeight="1"/>
-    <row r="404" ht="15.75" customHeight="1"/>
-    <row r="405" ht="15.75" customHeight="1"/>
-    <row r="406" ht="15.75" customHeight="1"/>
-    <row r="407" ht="15.75" customHeight="1"/>
-    <row r="408" ht="15.75" customHeight="1"/>
-    <row r="409" ht="15.75" customHeight="1"/>
-    <row r="410" ht="15.75" customHeight="1"/>
-    <row r="411" ht="15.75" customHeight="1"/>
-    <row r="412" ht="15.75" customHeight="1"/>
-    <row r="413" ht="15.75" customHeight="1"/>
-    <row r="414" ht="15.75" customHeight="1"/>
-    <row r="415" ht="15.75" customHeight="1"/>
-    <row r="416" ht="15.75" customHeight="1"/>
-    <row r="417" ht="15.75" customHeight="1"/>
-    <row r="418" ht="15.75" customHeight="1"/>
-    <row r="419" ht="15.75" customHeight="1"/>
-    <row r="420" ht="15.75" customHeight="1"/>
-    <row r="421" ht="15.75" customHeight="1"/>
-    <row r="422" ht="15.75" customHeight="1"/>
-    <row r="423" ht="15.75" customHeight="1"/>
-    <row r="424" ht="15.75" customHeight="1"/>
-    <row r="425" ht="15.75" customHeight="1"/>
-    <row r="426" ht="15.75" customHeight="1"/>
-    <row r="427" ht="15.75" customHeight="1"/>
-    <row r="428" ht="15.75" customHeight="1"/>
-    <row r="429" ht="15.75" customHeight="1"/>
-    <row r="430" ht="15.75" customHeight="1"/>
-    <row r="431" ht="15.75" customHeight="1"/>
-    <row r="432" ht="15.75" customHeight="1"/>
-    <row r="433" ht="15.75" customHeight="1"/>
-    <row r="434" ht="15.75" customHeight="1"/>
-    <row r="435" ht="15.75" customHeight="1"/>
-    <row r="436" ht="15.75" customHeight="1"/>
-    <row r="437" ht="15.75" customHeight="1"/>
-    <row r="438" ht="15.75" customHeight="1"/>
-    <row r="439" ht="15.75" customHeight="1"/>
-    <row r="440" ht="15.75" customHeight="1"/>
-    <row r="441" ht="15.75" customHeight="1"/>
-    <row r="442" ht="15.75" customHeight="1"/>
-    <row r="443" ht="15.75" customHeight="1"/>
-    <row r="444" ht="15.75" customHeight="1"/>
-    <row r="445" ht="15.75" customHeight="1"/>
-    <row r="446" ht="15.75" customHeight="1"/>
-    <row r="447" ht="15.75" customHeight="1"/>
-    <row r="448" ht="15.75" customHeight="1"/>
-    <row r="449" ht="15.75" customHeight="1"/>
-    <row r="450" ht="15.75" customHeight="1"/>
-    <row r="451" ht="15.75" customHeight="1"/>
-    <row r="452" ht="15.75" customHeight="1"/>
-    <row r="453" ht="15.75" customHeight="1"/>
-    <row r="454" ht="15.75" customHeight="1"/>
-    <row r="455" ht="15.75" customHeight="1"/>
-    <row r="456" ht="15.75" customHeight="1"/>
-    <row r="457" ht="15.75" customHeight="1"/>
-    <row r="458" ht="15.75" customHeight="1"/>
-    <row r="459" ht="15.75" customHeight="1"/>
-    <row r="460" ht="15.75" customHeight="1"/>
-    <row r="461" ht="15.75" customHeight="1"/>
-    <row r="462" ht="15.75" customHeight="1"/>
-    <row r="463" ht="15.75" customHeight="1"/>
-    <row r="464" ht="15.75" customHeight="1"/>
-    <row r="465" ht="15.75" customHeight="1"/>
-    <row r="466" ht="15.75" customHeight="1"/>
-    <row r="467" ht="15.75" customHeight="1"/>
-    <row r="468" ht="15.75" customHeight="1"/>
-    <row r="469" ht="15.75" customHeight="1"/>
-    <row r="470" ht="15.75" customHeight="1"/>
-    <row r="471" ht="15.75" customHeight="1"/>
-    <row r="472" ht="15.75" customHeight="1"/>
-    <row r="473" ht="15.75" customHeight="1"/>
-    <row r="474" ht="15.75" customHeight="1"/>
-    <row r="475" ht="15.75" customHeight="1"/>
-    <row r="476" ht="15.75" customHeight="1"/>
-    <row r="477" ht="15.75" customHeight="1"/>
-    <row r="478" ht="15.75" customHeight="1"/>
-    <row r="479" ht="15.75" customHeight="1"/>
-    <row r="480" ht="15.75" customHeight="1"/>
-    <row r="481" ht="15.75" customHeight="1"/>
-    <row r="482" ht="15.75" customHeight="1"/>
-    <row r="483" ht="15.75" customHeight="1"/>
-    <row r="484" ht="15.75" customHeight="1"/>
-    <row r="485" ht="15.75" customHeight="1"/>
-    <row r="486" ht="15.75" customHeight="1"/>
-    <row r="487" ht="15.75" customHeight="1"/>
-    <row r="488" ht="15.75" customHeight="1"/>
-    <row r="489" ht="15.75" customHeight="1"/>
-    <row r="490" ht="15.75" customHeight="1"/>
-    <row r="491" ht="15.75" customHeight="1"/>
-    <row r="492" ht="15.75" customHeight="1"/>
-    <row r="493" ht="15.75" customHeight="1"/>
-    <row r="494" ht="15.75" customHeight="1"/>
-    <row r="495" ht="15.75" customHeight="1"/>
-    <row r="496" ht="15.75" customHeight="1"/>
-    <row r="497" ht="15.75" customHeight="1"/>
-    <row r="498" ht="15.75" customHeight="1"/>
-    <row r="499" ht="15.75" customHeight="1"/>
-    <row r="500" ht="15.75" customHeight="1"/>
-    <row r="501" ht="15.75" customHeight="1"/>
-    <row r="502" ht="15.75" customHeight="1"/>
-    <row r="503" ht="15.75" customHeight="1"/>
-    <row r="504" ht="15.75" customHeight="1"/>
-    <row r="505" ht="15.75" customHeight="1"/>
-    <row r="506" ht="15.75" customHeight="1"/>
-    <row r="507" ht="15.75" customHeight="1"/>
-    <row r="508" ht="15.75" customHeight="1"/>
-    <row r="509" ht="15.75" customHeight="1"/>
-    <row r="510" ht="15.75" customHeight="1"/>
-    <row r="511" ht="15.75" customHeight="1"/>
-    <row r="512" ht="15.75" customHeight="1"/>
-    <row r="513" ht="15.75" customHeight="1"/>
-    <row r="514" ht="15.75" customHeight="1"/>
-    <row r="515" ht="15.75" customHeight="1"/>
-    <row r="516" ht="15.75" customHeight="1"/>
-    <row r="517" ht="15.75" customHeight="1"/>
-    <row r="518" ht="15.75" customHeight="1"/>
-    <row r="519" ht="15.75" customHeight="1"/>
-    <row r="520" ht="15.75" customHeight="1"/>
-    <row r="521" ht="15.75" customHeight="1"/>
-    <row r="522" ht="15.75" customHeight="1"/>
-    <row r="523" ht="15.75" customHeight="1"/>
-    <row r="524" ht="15.75" customHeight="1"/>
-    <row r="525" ht="15.75" customHeight="1"/>
-    <row r="526" ht="15.75" customHeight="1"/>
-    <row r="527" ht="15.75" customHeight="1"/>
-    <row r="528" ht="15.75" customHeight="1"/>
-    <row r="529" ht="15.75" customHeight="1"/>
-    <row r="530" ht="15.75" customHeight="1"/>
-    <row r="531" ht="15.75" customHeight="1"/>
-    <row r="532" ht="15.75" customHeight="1"/>
-    <row r="533" ht="15.75" customHeight="1"/>
-    <row r="534" ht="15.75" customHeight="1"/>
-    <row r="535" ht="15.75" customHeight="1"/>
-    <row r="536" ht="15.75" customHeight="1"/>
-    <row r="537" ht="15.75" customHeight="1"/>
-    <row r="538" ht="15.75" customHeight="1"/>
-    <row r="539" ht="15.75" customHeight="1"/>
-    <row r="540" ht="15.75" customHeight="1"/>
-    <row r="541" ht="15.75" customHeight="1"/>
-    <row r="542" ht="15.75" customHeight="1"/>
-    <row r="543" ht="15.75" customHeight="1"/>
-    <row r="544" ht="15.75" customHeight="1"/>
-    <row r="545" ht="15.75" customHeight="1"/>
-    <row r="546" ht="15.75" customHeight="1"/>
-    <row r="547" ht="15.75" customHeight="1"/>
-    <row r="548" ht="15.75" customHeight="1"/>
-    <row r="549" ht="15.75" customHeight="1"/>
-    <row r="550" ht="15.75" customHeight="1"/>
-    <row r="551" ht="15.75" customHeight="1"/>
-    <row r="552" ht="15.75" customHeight="1"/>
-    <row r="553" ht="15.75" customHeight="1"/>
-    <row r="554" ht="15.75" customHeight="1"/>
-    <row r="555" ht="15.75" customHeight="1"/>
-    <row r="556" ht="15.75" customHeight="1"/>
-    <row r="557" ht="15.75" customHeight="1"/>
-    <row r="558" ht="15.75" customHeight="1"/>
-    <row r="559" ht="15.75" customHeight="1"/>
-    <row r="560" ht="15.75" customHeight="1"/>
-    <row r="561" ht="15.75" customHeight="1"/>
-    <row r="562" ht="15.75" customHeight="1"/>
-    <row r="563" ht="15.75" customHeight="1"/>
-    <row r="564" ht="15.75" customHeight="1"/>
-    <row r="565" ht="15.75" customHeight="1"/>
-    <row r="566" ht="15.75" customHeight="1"/>
-    <row r="567" ht="15.75" customHeight="1"/>
-    <row r="568" ht="15.75" customHeight="1"/>
-    <row r="569" ht="15.75" customHeight="1"/>
-    <row r="570" ht="15.75" customHeight="1"/>
-    <row r="571" ht="15.75" customHeight="1"/>
-    <row r="572" ht="15.75" customHeight="1"/>
-    <row r="573" ht="15.75" customHeight="1"/>
-    <row r="574" ht="15.75" customHeight="1"/>
-    <row r="575" ht="15.75" customHeight="1"/>
-    <row r="576" ht="15.75" customHeight="1"/>
-    <row r="577" ht="15.75" customHeight="1"/>
-    <row r="578" ht="15.75" customHeight="1"/>
-    <row r="579" ht="15.75" customHeight="1"/>
-    <row r="580" ht="15.75" customHeight="1"/>
-    <row r="581" ht="15.75" customHeight="1"/>
-    <row r="582" ht="15.75" customHeight="1"/>
-    <row r="583" ht="15.75" customHeight="1"/>
-    <row r="584" ht="15.75" customHeight="1"/>
-    <row r="585" ht="15.75" customHeight="1"/>
-    <row r="586" ht="15.75" customHeight="1"/>
-    <row r="587" ht="15.75" customHeight="1"/>
-    <row r="588" ht="15.75" customHeight="1"/>
-    <row r="589" ht="15.75" customHeight="1"/>
-    <row r="590" ht="15.75" customHeight="1"/>
-    <row r="591" ht="15.75" customHeight="1"/>
-    <row r="592" ht="15.75" customHeight="1"/>
-    <row r="593" ht="15.75" customHeight="1"/>
-    <row r="594" ht="15.75" customHeight="1"/>
-    <row r="595" ht="15.75" customHeight="1"/>
-    <row r="596" ht="15.75" customHeight="1"/>
-    <row r="597" ht="15.75" customHeight="1"/>
-    <row r="598" ht="15.75" customHeight="1"/>
-    <row r="599" ht="15.75" customHeight="1"/>
-    <row r="600" ht="15.75" customHeight="1"/>
-    <row r="601" ht="15.75" customHeight="1"/>
-    <row r="602" ht="15.75" customHeight="1"/>
-    <row r="603" ht="15.75" customHeight="1"/>
-    <row r="604" ht="15.75" customHeight="1"/>
-    <row r="605" ht="15.75" customHeight="1"/>
-    <row r="606" ht="15.75" customHeight="1"/>
-    <row r="607" ht="15.75" customHeight="1"/>
-    <row r="608" ht="15.75" customHeight="1"/>
-    <row r="609" ht="15.75" customHeight="1"/>
-    <row r="610" ht="15.75" customHeight="1"/>
-    <row r="611" ht="15.75" customHeight="1"/>
-    <row r="612" ht="15.75" customHeight="1"/>
-    <row r="613" ht="15.75" customHeight="1"/>
-    <row r="614" ht="15.75" customHeight="1"/>
-    <row r="615" ht="15.75" customHeight="1"/>
-    <row r="616" ht="15.75" customHeight="1"/>
-    <row r="617" ht="15.75" customHeight="1"/>
-    <row r="618" ht="15.75" customHeight="1"/>
-    <row r="619" ht="15.75" customHeight="1"/>
-    <row r="620" ht="15.75" customHeight="1"/>
-    <row r="621" ht="15.75" customHeight="1"/>
-    <row r="622" ht="15.75" customHeight="1"/>
-    <row r="623" ht="15.75" customHeight="1"/>
-    <row r="624" ht="15.75" customHeight="1"/>
-    <row r="625" ht="15.75" customHeight="1"/>
-    <row r="626" ht="15.75" customHeight="1"/>
-    <row r="627" ht="15.75" customHeight="1"/>
-    <row r="628" ht="15.75" customHeight="1"/>
-    <row r="629" ht="15.75" customHeight="1"/>
-    <row r="630" ht="15.75" customHeight="1"/>
-    <row r="631" ht="15.75" customHeight="1"/>
-    <row r="632" ht="15.75" customHeight="1"/>
-    <row r="633" ht="15.75" customHeight="1"/>
-    <row r="634" ht="15.75" customHeight="1"/>
-    <row r="635" ht="15.75" customHeight="1"/>
-    <row r="636" ht="15.75" customHeight="1"/>
-    <row r="637" ht="15.75" customHeight="1"/>
-    <row r="638" ht="15.75" customHeight="1"/>
-    <row r="639" ht="15.75" customHeight="1"/>
-    <row r="640" ht="15.75" customHeight="1"/>
-    <row r="641" ht="15.75" customHeight="1"/>
-    <row r="642" ht="15.75" customHeight="1"/>
-    <row r="643" ht="15.75" customHeight="1"/>
-    <row r="644" ht="15.75" customHeight="1"/>
-    <row r="645" ht="15.75" customHeight="1"/>
-    <row r="646" ht="15.75" customHeight="1"/>
-    <row r="647" ht="15.75" customHeight="1"/>
-    <row r="648" ht="15.75" customHeight="1"/>
-    <row r="649" ht="15.75" customHeight="1"/>
-    <row r="650" ht="15.75" customHeight="1"/>
-    <row r="651" ht="15.75" customHeight="1"/>
-    <row r="652" ht="15.75" customHeight="1"/>
-    <row r="653" ht="15.75" customHeight="1"/>
-    <row r="654" ht="15.75" customHeight="1"/>
-    <row r="655" ht="15.75" customHeight="1"/>
-    <row r="656" ht="15.75" customHeight="1"/>
-    <row r="657" ht="15.75" customHeight="1"/>
-    <row r="658" ht="15.75" customHeight="1"/>
-    <row r="659" ht="15.75" customHeight="1"/>
-    <row r="660" ht="15.75" customHeight="1"/>
-    <row r="661" ht="15.75" customHeight="1"/>
-    <row r="662" ht="15.75" customHeight="1"/>
-    <row r="663" ht="15.75" customHeight="1"/>
-    <row r="664" ht="15.75" customHeight="1"/>
-    <row r="665" ht="15.75" customHeight="1"/>
-    <row r="666" ht="15.75" customHeight="1"/>
-    <row r="667" ht="15.75" customHeight="1"/>
-    <row r="668" ht="15.75" customHeight="1"/>
-    <row r="669" ht="15.75" customHeight="1"/>
-    <row r="670" ht="15.75" customHeight="1"/>
-    <row r="671" ht="15.75" customHeight="1"/>
-    <row r="672" ht="15.75" customHeight="1"/>
-    <row r="673" ht="15.75" customHeight="1"/>
-    <row r="674" ht="15.75" customHeight="1"/>
-    <row r="675" ht="15.75" customHeight="1"/>
-    <row r="676" ht="15.75" customHeight="1"/>
-    <row r="677" ht="15.75" customHeight="1"/>
-    <row r="678" ht="15.75" customHeight="1"/>
-    <row r="679" ht="15.75" customHeight="1"/>
-    <row r="680" ht="15.75" customHeight="1"/>
-    <row r="681" ht="15.75" customHeight="1"/>
-    <row r="682" ht="15.75" customHeight="1"/>
-    <row r="683" ht="15.75" customHeight="1"/>
-    <row r="684" ht="15.75" customHeight="1"/>
-    <row r="685" ht="15.75" customHeight="1"/>
-    <row r="686" ht="15.75" customHeight="1"/>
-    <row r="687" ht="15.75" customHeight="1"/>
-    <row r="688" ht="15.75" customHeight="1"/>
-    <row r="689" ht="15.75" customHeight="1"/>
-    <row r="690" ht="15.75" customHeight="1"/>
-    <row r="691" ht="15.75" customHeight="1"/>
-    <row r="692" ht="15.75" customHeight="1"/>
-    <row r="693" ht="15.75" customHeight="1"/>
-    <row r="694" ht="15.75" customHeight="1"/>
-    <row r="695" ht="15.75" customHeight="1"/>
-    <row r="696" ht="15.75" customHeight="1"/>
-    <row r="697" ht="15.75" customHeight="1"/>
-    <row r="698" ht="15.75" customHeight="1"/>
-    <row r="699" ht="15.75" customHeight="1"/>
-    <row r="700" ht="15.75" customHeight="1"/>
-    <row r="701" ht="15.75" customHeight="1"/>
-    <row r="702" ht="15.75" customHeight="1"/>
-    <row r="703" ht="15.75" customHeight="1"/>
-    <row r="704" ht="15.75" customHeight="1"/>
-    <row r="705" ht="15.75" customHeight="1"/>
-    <row r="706" ht="15.75" customHeight="1"/>
-    <row r="707" ht="15.75" customHeight="1"/>
-    <row r="708" ht="15.75" customHeight="1"/>
-    <row r="709" ht="15.75" customHeight="1"/>
-    <row r="710" ht="15.75" customHeight="1"/>
-    <row r="711" ht="15.75" customHeight="1"/>
-    <row r="712" ht="15.75" customHeight="1"/>
-    <row r="713" ht="15.75" customHeight="1"/>
-    <row r="714" ht="15.75" customHeight="1"/>
-    <row r="715" ht="15.75" customHeight="1"/>
-    <row r="716" ht="15.75" customHeight="1"/>
-    <row r="717" ht="15.75" customHeight="1"/>
-    <row r="718" ht="15.75" customHeight="1"/>
-    <row r="719" ht="15.75" customHeight="1"/>
-    <row r="720" ht="15.75" customHeight="1"/>
-    <row r="721" ht="15.75" customHeight="1"/>
-    <row r="722" ht="15.75" customHeight="1"/>
-    <row r="723" ht="15.75" customHeight="1"/>
-    <row r="724" ht="15.75" customHeight="1"/>
-    <row r="725" ht="15.75" customHeight="1"/>
-    <row r="726" ht="15.75" customHeight="1"/>
-    <row r="727" ht="15.75" customHeight="1"/>
-    <row r="728" ht="15.75" customHeight="1"/>
-    <row r="729" ht="15.75" customHeight="1"/>
-    <row r="730" ht="15.75" customHeight="1"/>
-    <row r="731" ht="15.75" customHeight="1"/>
-    <row r="732" ht="15.75" customHeight="1"/>
-    <row r="733" ht="15.75" customHeight="1"/>
-    <row r="734" ht="15.75" customHeight="1"/>
-    <row r="735" ht="15.75" customHeight="1"/>
-    <row r="736" ht="15.75" customHeight="1"/>
-    <row r="737" ht="15.75" customHeight="1"/>
-    <row r="738" ht="15.75" customHeight="1"/>
-    <row r="739" ht="15.75" customHeight="1"/>
-    <row r="740" ht="15.75" customHeight="1"/>
-    <row r="741" ht="15.75" customHeight="1"/>
-    <row r="742" ht="15.75" customHeight="1"/>
-    <row r="743" ht="15.75" customHeight="1"/>
-    <row r="744" ht="15.75" customHeight="1"/>
-    <row r="745" ht="15.75" customHeight="1"/>
-    <row r="746" ht="15.75" customHeight="1"/>
-    <row r="747" ht="15.75" customHeight="1"/>
-    <row r="748" ht="15.75" customHeight="1"/>
-    <row r="749" ht="15.75" customHeight="1"/>
-    <row r="750" ht="15.75" customHeight="1"/>
-    <row r="751" ht="15.75" customHeight="1"/>
-    <row r="752" ht="15.75" customHeight="1"/>
-    <row r="753" ht="15.75" customHeight="1"/>
-    <row r="754" ht="15.75" customHeight="1"/>
-    <row r="755" ht="15.75" customHeight="1"/>
-    <row r="756" ht="15.75" customHeight="1"/>
-    <row r="757" ht="15.75" customHeight="1"/>
-    <row r="758" ht="15.75" customHeight="1"/>
-    <row r="759" ht="15.75" customHeight="1"/>
-    <row r="760" ht="15.75" customHeight="1"/>
-    <row r="761" ht="15.75" customHeight="1"/>
-    <row r="762" ht="15.75" customHeight="1"/>
-    <row r="763" ht="15.75" customHeight="1"/>
-    <row r="764" ht="15.75" customHeight="1"/>
-    <row r="765" ht="15.75" customHeight="1"/>
-    <row r="766" ht="15.75" customHeight="1"/>
-    <row r="767" ht="15.75" customHeight="1"/>
-    <row r="768" ht="15.75" customHeight="1"/>
-    <row r="769" ht="15.75" customHeight="1"/>
-    <row r="770" ht="15.75" customHeight="1"/>
-    <row r="771" ht="15.75" customHeight="1"/>
-    <row r="772" ht="15.75" customHeight="1"/>
-    <row r="773" ht="15.75" customHeight="1"/>
-    <row r="774" ht="15.75" customHeight="1"/>
-    <row r="775" ht="15.75" customHeight="1"/>
-    <row r="776" ht="15.75" customHeight="1"/>
-    <row r="777" ht="15.75" customHeight="1"/>
-    <row r="778" ht="15.75" customHeight="1"/>
-    <row r="779" ht="15.75" customHeight="1"/>
-    <row r="780" ht="15.75" customHeight="1"/>
-    <row r="781" ht="15.75" customHeight="1"/>
-    <row r="782" ht="15.75" customHeight="1"/>
-    <row r="783" ht="15.75" customHeight="1"/>
-    <row r="784" ht="15.75" customHeight="1"/>
-    <row r="785" ht="15.75" customHeight="1"/>
-    <row r="786" ht="15.75" customHeight="1"/>
-    <row r="787" ht="15.75" customHeight="1"/>
-    <row r="788" ht="15.75" customHeight="1"/>
-    <row r="789" ht="15.75" customHeight="1"/>
-    <row r="790" ht="15.75" customHeight="1"/>
-    <row r="791" ht="15.75" customHeight="1"/>
-    <row r="792" ht="15.75" customHeight="1"/>
-    <row r="793" ht="15.75" customHeight="1"/>
-    <row r="794" ht="15.75" customHeight="1"/>
-    <row r="795" ht="15.75" customHeight="1"/>
-    <row r="796" ht="15.75" customHeight="1"/>
-    <row r="797" ht="15.75" customHeight="1"/>
-    <row r="798" ht="15.75" customHeight="1"/>
-    <row r="799" ht="15.75" customHeight="1"/>
-    <row r="800" ht="15.75" customHeight="1"/>
-    <row r="801" ht="15.75" customHeight="1"/>
-    <row r="802" ht="15.75" customHeight="1"/>
-    <row r="803" ht="15.75" customHeight="1"/>
-    <row r="804" ht="15.75" customHeight="1"/>
-    <row r="805" ht="15.75" customHeight="1"/>
-    <row r="806" ht="15.75" customHeight="1"/>
-    <row r="807" ht="15.75" customHeight="1"/>
-    <row r="808" ht="15.75" customHeight="1"/>
-    <row r="809" ht="15.75" customHeight="1"/>
-    <row r="810" ht="15.75" customHeight="1"/>
-    <row r="811" ht="15.75" customHeight="1"/>
-    <row r="812" ht="15.75" customHeight="1"/>
-    <row r="813" ht="15.75" customHeight="1"/>
-    <row r="814" ht="15.75" customHeight="1"/>
-    <row r="815" ht="15.75" customHeight="1"/>
-    <row r="816" ht="15.75" customHeight="1"/>
-    <row r="817" ht="15.75" customHeight="1"/>
-    <row r="818" ht="15.75" customHeight="1"/>
-    <row r="819" ht="15.75" customHeight="1"/>
-    <row r="820" ht="15.75" customHeight="1"/>
-    <row r="821" ht="15.75" customHeight="1"/>
-    <row r="822" ht="15.75" customHeight="1"/>
-    <row r="823" ht="15.75" customHeight="1"/>
-    <row r="824" ht="15.75" customHeight="1"/>
-    <row r="825" ht="15.75" customHeight="1"/>
-    <row r="826" ht="15.75" customHeight="1"/>
-    <row r="827" ht="15.75" customHeight="1"/>
-    <row r="828" ht="15.75" customHeight="1"/>
-    <row r="829" ht="15.75" customHeight="1"/>
-    <row r="830" ht="15.75" customHeight="1"/>
-    <row r="831" ht="15.75" customHeight="1"/>
-    <row r="832" ht="15.75" customHeight="1"/>
-    <row r="833" ht="15.75" customHeight="1"/>
-    <row r="834" ht="15.75" customHeight="1"/>
-    <row r="835" ht="15.75" customHeight="1"/>
-    <row r="836" ht="15.75" customHeight="1"/>
-    <row r="837" ht="15.75" customHeight="1"/>
-    <row r="838" ht="15.75" customHeight="1"/>
-    <row r="839" ht="15.75" customHeight="1"/>
-    <row r="840" ht="15.75" customHeight="1"/>
-    <row r="841" ht="15.75" customHeight="1"/>
-    <row r="842" ht="15.75" customHeight="1"/>
-    <row r="843" ht="15.75" customHeight="1"/>
-    <row r="844" ht="15.75" customHeight="1"/>
-    <row r="845" ht="15.75" customHeight="1"/>
-    <row r="846" ht="15.75" customHeight="1"/>
-    <row r="847" ht="15.75" customHeight="1"/>
-    <row r="848" ht="15.75" customHeight="1"/>
-    <row r="849" ht="15.75" customHeight="1"/>
-    <row r="850" ht="15.75" customHeight="1"/>
-    <row r="851" ht="15.75" customHeight="1"/>
-    <row r="852" ht="15.75" customHeight="1"/>
-    <row r="853" ht="15.75" customHeight="1"/>
-    <row r="854" ht="15.75" customHeight="1"/>
-    <row r="855" ht="15.75" customHeight="1"/>
-    <row r="856" ht="15.75" customHeight="1"/>
-    <row r="857" ht="15.75" customHeight="1"/>
-    <row r="858" ht="15.75" customHeight="1"/>
-    <row r="859" ht="15.75" customHeight="1"/>
-    <row r="860" ht="15.75" customHeight="1"/>
-    <row r="861" ht="15.75" customHeight="1"/>
-    <row r="862" ht="15.75" customHeight="1"/>
-    <row r="863" ht="15.75" customHeight="1"/>
-    <row r="864" ht="15.75" customHeight="1"/>
-    <row r="865" ht="15.75" customHeight="1"/>
-    <row r="866" ht="15.75" customHeight="1"/>
-    <row r="867" ht="15.75" customHeight="1"/>
-    <row r="868" ht="15.75" customHeight="1"/>
-    <row r="869" ht="15.75" customHeight="1"/>
-    <row r="870" ht="15.75" customHeight="1"/>
-    <row r="871" ht="15.75" customHeight="1"/>
-    <row r="872" ht="15.75" customHeight="1"/>
-    <row r="873" ht="15.75" customHeight="1"/>
-    <row r="874" ht="15.75" customHeight="1"/>
-    <row r="875" ht="15.75" customHeight="1"/>
-    <row r="876" ht="15.75" customHeight="1"/>
-    <row r="877" ht="15.75" customHeight="1"/>
-    <row r="878" ht="15.75" customHeight="1"/>
-    <row r="879" ht="15.75" customHeight="1"/>
-    <row r="880" ht="15.75" customHeight="1"/>
-    <row r="881" ht="15.75" customHeight="1"/>
-    <row r="882" ht="15.75" customHeight="1"/>
-    <row r="883" ht="15.75" customHeight="1"/>
-    <row r="884" ht="15.75" customHeight="1"/>
-    <row r="885" ht="15.75" customHeight="1"/>
-    <row r="886" ht="15.75" customHeight="1"/>
-    <row r="887" ht="15.75" customHeight="1"/>
-    <row r="888" ht="15.75" customHeight="1"/>
-    <row r="889" ht="15.75" customHeight="1"/>
-    <row r="890" ht="15.75" customHeight="1"/>
-    <row r="891" ht="15.75" customHeight="1"/>
-    <row r="892" ht="15.75" customHeight="1"/>
-    <row r="893" ht="15.75" customHeight="1"/>
-    <row r="894" ht="15.75" customHeight="1"/>
-    <row r="895" ht="15.75" customHeight="1"/>
-    <row r="896" ht="15.75" customHeight="1"/>
-    <row r="897" ht="15.75" customHeight="1"/>
-    <row r="898" ht="15.75" customHeight="1"/>
-    <row r="899" ht="15.75" customHeight="1"/>
-    <row r="900" ht="15.75" customHeight="1"/>
-    <row r="901" ht="15.75" customHeight="1"/>
-    <row r="902" ht="15.75" customHeight="1"/>
-    <row r="903" ht="15.75" customHeight="1"/>
-    <row r="904" ht="15.75" customHeight="1"/>
-    <row r="905" ht="15.75" customHeight="1"/>
-    <row r="906" ht="15.75" customHeight="1"/>
-    <row r="907" ht="15.75" customHeight="1"/>
-    <row r="908" ht="15.75" customHeight="1"/>
-    <row r="909" ht="15.75" customHeight="1"/>
-    <row r="910" ht="15.75" customHeight="1"/>
-    <row r="911" ht="15.75" customHeight="1"/>
-    <row r="912" ht="15.75" customHeight="1"/>
-    <row r="913" ht="15.75" customHeight="1"/>
-    <row r="914" ht="15.75" customHeight="1"/>
-    <row r="915" ht="15.75" customHeight="1"/>
-    <row r="916" ht="15.75" customHeight="1"/>
-    <row r="917" ht="15.75" customHeight="1"/>
-    <row r="918" ht="15.75" customHeight="1"/>
-    <row r="919" ht="15.75" customHeight="1"/>
-    <row r="920" ht="15.75" customHeight="1"/>
-    <row r="921" ht="15.75" customHeight="1"/>
-    <row r="922" ht="15.75" customHeight="1"/>
-    <row r="923" ht="15.75" customHeight="1"/>
-    <row r="924" ht="15.75" customHeight="1"/>
-    <row r="925" ht="15.75" customHeight="1"/>
-    <row r="926" ht="15.75" customHeight="1"/>
-    <row r="927" ht="15.75" customHeight="1"/>
-    <row r="928" ht="15.75" customHeight="1"/>
-    <row r="929" ht="15.75" customHeight="1"/>
-    <row r="930" ht="15.75" customHeight="1"/>
-    <row r="931" ht="15.75" customHeight="1"/>
-    <row r="932" ht="15.75" customHeight="1"/>
-    <row r="933" ht="15.75" customHeight="1"/>
-    <row r="934" ht="15.75" customHeight="1"/>
-    <row r="935" ht="15.75" customHeight="1"/>
-    <row r="936" ht="15.75" customHeight="1"/>
-    <row r="937" ht="15.75" customHeight="1"/>
-    <row r="938" ht="15.75" customHeight="1"/>
-    <row r="939" ht="15.75" customHeight="1"/>
-    <row r="940" ht="15.75" customHeight="1"/>
-    <row r="941" ht="15.75" customHeight="1"/>
-    <row r="942" ht="15.75" customHeight="1"/>
-    <row r="943" ht="15.75" customHeight="1"/>
-    <row r="944" ht="15.75" customHeight="1"/>
-    <row r="945" ht="15.75" customHeight="1"/>
-    <row r="946" ht="15.75" customHeight="1"/>
-    <row r="947" ht="15.75" customHeight="1"/>
-    <row r="948" ht="15.75" customHeight="1"/>
-    <row r="949" ht="15.75" customHeight="1"/>
-    <row r="950" ht="15.75" customHeight="1"/>
-    <row r="951" ht="15.75" customHeight="1"/>
-    <row r="952" ht="15.75" customHeight="1"/>
-    <row r="953" ht="15.75" customHeight="1"/>
-    <row r="954" ht="15.75" customHeight="1"/>
-    <row r="955" ht="15.75" customHeight="1"/>
-    <row r="956" ht="15.75" customHeight="1"/>
-    <row r="957" ht="15.75" customHeight="1"/>
-    <row r="958" ht="15.75" customHeight="1"/>
-    <row r="959" ht="15.75" customHeight="1"/>
-    <row r="960" ht="15.75" customHeight="1"/>
-    <row r="961" ht="15.75" customHeight="1"/>
-    <row r="962" ht="15.75" customHeight="1"/>
-    <row r="963" ht="15.75" customHeight="1"/>
-    <row r="964" ht="15.75" customHeight="1"/>
-    <row r="965" ht="15.75" customHeight="1"/>
-    <row r="966" ht="15.75" customHeight="1"/>
-    <row r="967" ht="15.75" customHeight="1"/>
-    <row r="968" ht="15.75" customHeight="1"/>
-    <row r="969" ht="15.75" customHeight="1"/>
-    <row r="970" ht="15.75" customHeight="1"/>
-    <row r="971" ht="15.75" customHeight="1"/>
-    <row r="972" ht="15.75" customHeight="1"/>
-    <row r="973" ht="15.75" customHeight="1"/>
-    <row r="974" ht="15.75" customHeight="1"/>
-    <row r="975" ht="15.75" customHeight="1"/>
-    <row r="976" ht="15.75" customHeight="1"/>
-    <row r="977" ht="15.75" customHeight="1"/>
-    <row r="978" ht="15.75" customHeight="1"/>
-    <row r="979" ht="15.75" customHeight="1"/>
-    <row r="980" ht="15.75" customHeight="1"/>
-    <row r="981" ht="15.75" customHeight="1"/>
-    <row r="982" ht="15.75" customHeight="1"/>
-    <row r="983" ht="15.75" customHeight="1"/>
-    <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
-    <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
+      <c r="AA220" s="1"/>
+    </row>
+    <row r="221" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="222" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="223" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="224" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.984027777777778" footer="0.0" header="0.0" left="0.747916666666667" right="0.747916666666667" top="0.984027777777778"/>
+  <pageMargins left="0.74791666666666701" right="0.74791666666666701" top="0.98402777777777795" bottom="0.98402777777777795" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix import tape and external quality report
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportExternalQualityReportTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportExternalQualityReportTemplate.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Tên rút gọn</t>
   </si>
@@ -338,24 +338,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AA1000"/>
+  <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" customWidth="1"/>
-    <col min="5" max="6" width="12.5703125" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" customWidth="1"/>
-    <col min="10" max="10" width="19.85546875" customWidth="1"/>
-    <col min="12" max="12" width="23.5703125" customWidth="1"/>
-    <col min="13" max="13" width="42.5703125" customWidth="1"/>
-    <col min="14" max="14" width="38.28515625" customWidth="1"/>
-    <col min="15" max="15" width="10.28515625" customWidth="1"/>
+    <col min="4" max="5" width="12.5703125" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="9" max="9" width="19.85546875" customWidth="1"/>
+    <col min="11" max="11" width="23.5703125" customWidth="1"/>
+    <col min="12" max="12" width="42.5703125" customWidth="1"/>
+    <col min="13" max="13" width="38.28515625" customWidth="1"/>
+    <col min="14" max="14" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -382,9 +381,8 @@
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
-      <c r="AA1" s="1"/>
-    </row>
-    <row r="2" spans="1:27" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:26" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -395,41 +393,39 @@
         <v>2</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="L2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="M2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="O2" s="1"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -441,9 +437,8 @@
       <c r="X2" s="1"/>
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
-      <c r="AA2" s="1"/>
-    </row>
-    <row r="3" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -470,9 +465,8 @@
       <c r="X3" s="1"/>
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
-      <c r="AA3" s="1"/>
-    </row>
-    <row r="4" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -499,9 +493,8 @@
       <c r="X4" s="1"/>
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
-      <c r="AA4" s="1"/>
-    </row>
-    <row r="5" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -528,9 +521,8 @@
       <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
-      <c r="AA5" s="1"/>
-    </row>
-    <row r="6" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -557,9 +549,8 @@
       <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
-      <c r="AA6" s="1"/>
-    </row>
-    <row r="7" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -586,9 +577,8 @@
       <c r="X7" s="1"/>
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
-      <c r="AA7" s="1"/>
-    </row>
-    <row r="8" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -615,9 +605,8 @@
       <c r="X8" s="1"/>
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
-      <c r="AA8" s="1"/>
-    </row>
-    <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -644,9 +633,8 @@
       <c r="X9" s="1"/>
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
-      <c r="AA9" s="1"/>
-    </row>
-    <row r="10" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -673,9 +661,8 @@
       <c r="X10" s="1"/>
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
-      <c r="AA10" s="1"/>
-    </row>
-    <row r="11" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -702,9 +689,8 @@
       <c r="X11" s="1"/>
       <c r="Y11" s="1"/>
       <c r="Z11" s="1"/>
-      <c r="AA11" s="1"/>
-    </row>
-    <row r="12" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -731,9 +717,8 @@
       <c r="X12" s="1"/>
       <c r="Y12" s="1"/>
       <c r="Z12" s="1"/>
-      <c r="AA12" s="1"/>
-    </row>
-    <row r="13" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -760,9 +745,8 @@
       <c r="X13" s="1"/>
       <c r="Y13" s="1"/>
       <c r="Z13" s="1"/>
-      <c r="AA13" s="1"/>
-    </row>
-    <row r="14" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -789,9 +773,8 @@
       <c r="X14" s="1"/>
       <c r="Y14" s="1"/>
       <c r="Z14" s="1"/>
-      <c r="AA14" s="1"/>
-    </row>
-    <row r="15" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -818,9 +801,8 @@
       <c r="X15" s="1"/>
       <c r="Y15" s="1"/>
       <c r="Z15" s="1"/>
-      <c r="AA15" s="1"/>
-    </row>
-    <row r="16" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -847,9 +829,8 @@
       <c r="X16" s="1"/>
       <c r="Y16" s="1"/>
       <c r="Z16" s="1"/>
-      <c r="AA16" s="1"/>
-    </row>
-    <row r="17" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -876,9 +857,8 @@
       <c r="X17" s="1"/>
       <c r="Y17" s="1"/>
       <c r="Z17" s="1"/>
-      <c r="AA17" s="1"/>
-    </row>
-    <row r="18" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -905,9 +885,8 @@
       <c r="X18" s="1"/>
       <c r="Y18" s="1"/>
       <c r="Z18" s="1"/>
-      <c r="AA18" s="1"/>
-    </row>
-    <row r="19" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -934,9 +913,8 @@
       <c r="X19" s="1"/>
       <c r="Y19" s="1"/>
       <c r="Z19" s="1"/>
-      <c r="AA19" s="1"/>
-    </row>
-    <row r="20" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -963,9 +941,8 @@
       <c r="X20" s="1"/>
       <c r="Y20" s="1"/>
       <c r="Z20" s="1"/>
-      <c r="AA20" s="1"/>
-    </row>
-    <row r="21" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -992,9 +969,8 @@
       <c r="X21" s="1"/>
       <c r="Y21" s="1"/>
       <c r="Z21" s="1"/>
-      <c r="AA21" s="1"/>
-    </row>
-    <row r="22" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -1021,9 +997,8 @@
       <c r="X22" s="1"/>
       <c r="Y22" s="1"/>
       <c r="Z22" s="1"/>
-      <c r="AA22" s="1"/>
-    </row>
-    <row r="23" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1050,9 +1025,8 @@
       <c r="X23" s="1"/>
       <c r="Y23" s="1"/>
       <c r="Z23" s="1"/>
-      <c r="AA23" s="1"/>
-    </row>
-    <row r="24" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1079,9 +1053,8 @@
       <c r="X24" s="1"/>
       <c r="Y24" s="1"/>
       <c r="Z24" s="1"/>
-      <c r="AA24" s="1"/>
-    </row>
-    <row r="25" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1108,9 +1081,8 @@
       <c r="X25" s="1"/>
       <c r="Y25" s="1"/>
       <c r="Z25" s="1"/>
-      <c r="AA25" s="1"/>
-    </row>
-    <row r="26" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1137,9 +1109,8 @@
       <c r="X26" s="1"/>
       <c r="Y26" s="1"/>
       <c r="Z26" s="1"/>
-      <c r="AA26" s="1"/>
-    </row>
-    <row r="27" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1166,9 +1137,8 @@
       <c r="X27" s="1"/>
       <c r="Y27" s="1"/>
       <c r="Z27" s="1"/>
-      <c r="AA27" s="1"/>
-    </row>
-    <row r="28" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1195,9 +1165,8 @@
       <c r="X28" s="1"/>
       <c r="Y28" s="1"/>
       <c r="Z28" s="1"/>
-      <c r="AA28" s="1"/>
-    </row>
-    <row r="29" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1224,9 +1193,8 @@
       <c r="X29" s="1"/>
       <c r="Y29" s="1"/>
       <c r="Z29" s="1"/>
-      <c r="AA29" s="1"/>
-    </row>
-    <row r="30" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -1253,9 +1221,8 @@
       <c r="X30" s="1"/>
       <c r="Y30" s="1"/>
       <c r="Z30" s="1"/>
-      <c r="AA30" s="1"/>
-    </row>
-    <row r="31" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1282,9 +1249,8 @@
       <c r="X31" s="1"/>
       <c r="Y31" s="1"/>
       <c r="Z31" s="1"/>
-      <c r="AA31" s="1"/>
-    </row>
-    <row r="32" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -1311,9 +1277,8 @@
       <c r="X32" s="1"/>
       <c r="Y32" s="1"/>
       <c r="Z32" s="1"/>
-      <c r="AA32" s="1"/>
-    </row>
-    <row r="33" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -1340,9 +1305,8 @@
       <c r="X33" s="1"/>
       <c r="Y33" s="1"/>
       <c r="Z33" s="1"/>
-      <c r="AA33" s="1"/>
-    </row>
-    <row r="34" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -1369,9 +1333,8 @@
       <c r="X34" s="1"/>
       <c r="Y34" s="1"/>
       <c r="Z34" s="1"/>
-      <c r="AA34" s="1"/>
-    </row>
-    <row r="35" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -1398,9 +1361,8 @@
       <c r="X35" s="1"/>
       <c r="Y35" s="1"/>
       <c r="Z35" s="1"/>
-      <c r="AA35" s="1"/>
-    </row>
-    <row r="36" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -1427,9 +1389,8 @@
       <c r="X36" s="1"/>
       <c r="Y36" s="1"/>
       <c r="Z36" s="1"/>
-      <c r="AA36" s="1"/>
-    </row>
-    <row r="37" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -1456,9 +1417,8 @@
       <c r="X37" s="1"/>
       <c r="Y37" s="1"/>
       <c r="Z37" s="1"/>
-      <c r="AA37" s="1"/>
-    </row>
-    <row r="38" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -1485,9 +1445,8 @@
       <c r="X38" s="1"/>
       <c r="Y38" s="1"/>
       <c r="Z38" s="1"/>
-      <c r="AA38" s="1"/>
-    </row>
-    <row r="39" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -1514,9 +1473,8 @@
       <c r="X39" s="1"/>
       <c r="Y39" s="1"/>
       <c r="Z39" s="1"/>
-      <c r="AA39" s="1"/>
-    </row>
-    <row r="40" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -1543,9 +1501,8 @@
       <c r="X40" s="1"/>
       <c r="Y40" s="1"/>
       <c r="Z40" s="1"/>
-      <c r="AA40" s="1"/>
-    </row>
-    <row r="41" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -1572,9 +1529,8 @@
       <c r="X41" s="1"/>
       <c r="Y41" s="1"/>
       <c r="Z41" s="1"/>
-      <c r="AA41" s="1"/>
-    </row>
-    <row r="42" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -1601,9 +1557,8 @@
       <c r="X42" s="1"/>
       <c r="Y42" s="1"/>
       <c r="Z42" s="1"/>
-      <c r="AA42" s="1"/>
-    </row>
-    <row r="43" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -1630,9 +1585,8 @@
       <c r="X43" s="1"/>
       <c r="Y43" s="1"/>
       <c r="Z43" s="1"/>
-      <c r="AA43" s="1"/>
-    </row>
-    <row r="44" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -1659,9 +1613,8 @@
       <c r="X44" s="1"/>
       <c r="Y44" s="1"/>
       <c r="Z44" s="1"/>
-      <c r="AA44" s="1"/>
-    </row>
-    <row r="45" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -1688,9 +1641,8 @@
       <c r="X45" s="1"/>
       <c r="Y45" s="1"/>
       <c r="Z45" s="1"/>
-      <c r="AA45" s="1"/>
-    </row>
-    <row r="46" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -1717,9 +1669,8 @@
       <c r="X46" s="1"/>
       <c r="Y46" s="1"/>
       <c r="Z46" s="1"/>
-      <c r="AA46" s="1"/>
-    </row>
-    <row r="47" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -1746,9 +1697,8 @@
       <c r="X47" s="1"/>
       <c r="Y47" s="1"/>
       <c r="Z47" s="1"/>
-      <c r="AA47" s="1"/>
-    </row>
-    <row r="48" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -1775,9 +1725,8 @@
       <c r="X48" s="1"/>
       <c r="Y48" s="1"/>
       <c r="Z48" s="1"/>
-      <c r="AA48" s="1"/>
-    </row>
-    <row r="49" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -1804,9 +1753,8 @@
       <c r="X49" s="1"/>
       <c r="Y49" s="1"/>
       <c r="Z49" s="1"/>
-      <c r="AA49" s="1"/>
-    </row>
-    <row r="50" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -1833,9 +1781,8 @@
       <c r="X50" s="1"/>
       <c r="Y50" s="1"/>
       <c r="Z50" s="1"/>
-      <c r="AA50" s="1"/>
-    </row>
-    <row r="51" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -1862,9 +1809,8 @@
       <c r="X51" s="1"/>
       <c r="Y51" s="1"/>
       <c r="Z51" s="1"/>
-      <c r="AA51" s="1"/>
-    </row>
-    <row r="52" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -1891,9 +1837,8 @@
       <c r="X52" s="1"/>
       <c r="Y52" s="1"/>
       <c r="Z52" s="1"/>
-      <c r="AA52" s="1"/>
-    </row>
-    <row r="53" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -1920,9 +1865,8 @@
       <c r="X53" s="1"/>
       <c r="Y53" s="1"/>
       <c r="Z53" s="1"/>
-      <c r="AA53" s="1"/>
-    </row>
-    <row r="54" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -1949,9 +1893,8 @@
       <c r="X54" s="1"/>
       <c r="Y54" s="1"/>
       <c r="Z54" s="1"/>
-      <c r="AA54" s="1"/>
-    </row>
-    <row r="55" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -1978,9 +1921,8 @@
       <c r="X55" s="1"/>
       <c r="Y55" s="1"/>
       <c r="Z55" s="1"/>
-      <c r="AA55" s="1"/>
-    </row>
-    <row r="56" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -2007,9 +1949,8 @@
       <c r="X56" s="1"/>
       <c r="Y56" s="1"/>
       <c r="Z56" s="1"/>
-      <c r="AA56" s="1"/>
-    </row>
-    <row r="57" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -2036,9 +1977,8 @@
       <c r="X57" s="1"/>
       <c r="Y57" s="1"/>
       <c r="Z57" s="1"/>
-      <c r="AA57" s="1"/>
-    </row>
-    <row r="58" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -2065,9 +2005,8 @@
       <c r="X58" s="1"/>
       <c r="Y58" s="1"/>
       <c r="Z58" s="1"/>
-      <c r="AA58" s="1"/>
-    </row>
-    <row r="59" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -2094,9 +2033,8 @@
       <c r="X59" s="1"/>
       <c r="Y59" s="1"/>
       <c r="Z59" s="1"/>
-      <c r="AA59" s="1"/>
-    </row>
-    <row r="60" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -2123,9 +2061,8 @@
       <c r="X60" s="1"/>
       <c r="Y60" s="1"/>
       <c r="Z60" s="1"/>
-      <c r="AA60" s="1"/>
-    </row>
-    <row r="61" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -2152,9 +2089,8 @@
       <c r="X61" s="1"/>
       <c r="Y61" s="1"/>
       <c r="Z61" s="1"/>
-      <c r="AA61" s="1"/>
-    </row>
-    <row r="62" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
@@ -2181,9 +2117,8 @@
       <c r="X62" s="1"/>
       <c r="Y62" s="1"/>
       <c r="Z62" s="1"/>
-      <c r="AA62" s="1"/>
-    </row>
-    <row r="63" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
@@ -2210,9 +2145,8 @@
       <c r="X63" s="1"/>
       <c r="Y63" s="1"/>
       <c r="Z63" s="1"/>
-      <c r="AA63" s="1"/>
-    </row>
-    <row r="64" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
@@ -2239,9 +2173,8 @@
       <c r="X64" s="1"/>
       <c r="Y64" s="1"/>
       <c r="Z64" s="1"/>
-      <c r="AA64" s="1"/>
-    </row>
-    <row r="65" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
@@ -2268,9 +2201,8 @@
       <c r="X65" s="1"/>
       <c r="Y65" s="1"/>
       <c r="Z65" s="1"/>
-      <c r="AA65" s="1"/>
-    </row>
-    <row r="66" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
@@ -2297,9 +2229,8 @@
       <c r="X66" s="1"/>
       <c r="Y66" s="1"/>
       <c r="Z66" s="1"/>
-      <c r="AA66" s="1"/>
-    </row>
-    <row r="67" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -2326,9 +2257,8 @@
       <c r="X67" s="1"/>
       <c r="Y67" s="1"/>
       <c r="Z67" s="1"/>
-      <c r="AA67" s="1"/>
-    </row>
-    <row r="68" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -2355,9 +2285,8 @@
       <c r="X68" s="1"/>
       <c r="Y68" s="1"/>
       <c r="Z68" s="1"/>
-      <c r="AA68" s="1"/>
-    </row>
-    <row r="69" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="69" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
@@ -2384,9 +2313,8 @@
       <c r="X69" s="1"/>
       <c r="Y69" s="1"/>
       <c r="Z69" s="1"/>
-      <c r="AA69" s="1"/>
-    </row>
-    <row r="70" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="70" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
@@ -2413,9 +2341,8 @@
       <c r="X70" s="1"/>
       <c r="Y70" s="1"/>
       <c r="Z70" s="1"/>
-      <c r="AA70" s="1"/>
-    </row>
-    <row r="71" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
@@ -2442,9 +2369,8 @@
       <c r="X71" s="1"/>
       <c r="Y71" s="1"/>
       <c r="Z71" s="1"/>
-      <c r="AA71" s="1"/>
-    </row>
-    <row r="72" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
@@ -2471,9 +2397,8 @@
       <c r="X72" s="1"/>
       <c r="Y72" s="1"/>
       <c r="Z72" s="1"/>
-      <c r="AA72" s="1"/>
-    </row>
-    <row r="73" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
@@ -2500,9 +2425,8 @@
       <c r="X73" s="1"/>
       <c r="Y73" s="1"/>
       <c r="Z73" s="1"/>
-      <c r="AA73" s="1"/>
-    </row>
-    <row r="74" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="74" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
@@ -2529,9 +2453,8 @@
       <c r="X74" s="1"/>
       <c r="Y74" s="1"/>
       <c r="Z74" s="1"/>
-      <c r="AA74" s="1"/>
-    </row>
-    <row r="75" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="75" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
@@ -2558,9 +2481,8 @@
       <c r="X75" s="1"/>
       <c r="Y75" s="1"/>
       <c r="Z75" s="1"/>
-      <c r="AA75" s="1"/>
-    </row>
-    <row r="76" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
@@ -2587,9 +2509,8 @@
       <c r="X76" s="1"/>
       <c r="Y76" s="1"/>
       <c r="Z76" s="1"/>
-      <c r="AA76" s="1"/>
-    </row>
-    <row r="77" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="77" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
@@ -2616,9 +2537,8 @@
       <c r="X77" s="1"/>
       <c r="Y77" s="1"/>
       <c r="Z77" s="1"/>
-      <c r="AA77" s="1"/>
-    </row>
-    <row r="78" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
@@ -2645,9 +2565,8 @@
       <c r="X78" s="1"/>
       <c r="Y78" s="1"/>
       <c r="Z78" s="1"/>
-      <c r="AA78" s="1"/>
-    </row>
-    <row r="79" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="79" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -2674,9 +2593,8 @@
       <c r="X79" s="1"/>
       <c r="Y79" s="1"/>
       <c r="Z79" s="1"/>
-      <c r="AA79" s="1"/>
-    </row>
-    <row r="80" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="80" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
@@ -2703,9 +2621,8 @@
       <c r="X80" s="1"/>
       <c r="Y80" s="1"/>
       <c r="Z80" s="1"/>
-      <c r="AA80" s="1"/>
-    </row>
-    <row r="81" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="81" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
@@ -2732,9 +2649,8 @@
       <c r="X81" s="1"/>
       <c r="Y81" s="1"/>
       <c r="Z81" s="1"/>
-      <c r="AA81" s="1"/>
-    </row>
-    <row r="82" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -2761,9 +2677,8 @@
       <c r="X82" s="1"/>
       <c r="Y82" s="1"/>
       <c r="Z82" s="1"/>
-      <c r="AA82" s="1"/>
-    </row>
-    <row r="83" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="83" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
@@ -2790,9 +2705,8 @@
       <c r="X83" s="1"/>
       <c r="Y83" s="1"/>
       <c r="Z83" s="1"/>
-      <c r="AA83" s="1"/>
-    </row>
-    <row r="84" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="84" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -2819,9 +2733,8 @@
       <c r="X84" s="1"/>
       <c r="Y84" s="1"/>
       <c r="Z84" s="1"/>
-      <c r="AA84" s="1"/>
-    </row>
-    <row r="85" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="85" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
@@ -2848,9 +2761,8 @@
       <c r="X85" s="1"/>
       <c r="Y85" s="1"/>
       <c r="Z85" s="1"/>
-      <c r="AA85" s="1"/>
-    </row>
-    <row r="86" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="86" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
@@ -2877,9 +2789,8 @@
       <c r="X86" s="1"/>
       <c r="Y86" s="1"/>
       <c r="Z86" s="1"/>
-      <c r="AA86" s="1"/>
-    </row>
-    <row r="87" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="87" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
@@ -2906,9 +2817,8 @@
       <c r="X87" s="1"/>
       <c r="Y87" s="1"/>
       <c r="Z87" s="1"/>
-      <c r="AA87" s="1"/>
-    </row>
-    <row r="88" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
@@ -2935,9 +2845,8 @@
       <c r="X88" s="1"/>
       <c r="Y88" s="1"/>
       <c r="Z88" s="1"/>
-      <c r="AA88" s="1"/>
-    </row>
-    <row r="89" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
@@ -2964,9 +2873,8 @@
       <c r="X89" s="1"/>
       <c r="Y89" s="1"/>
       <c r="Z89" s="1"/>
-      <c r="AA89" s="1"/>
-    </row>
-    <row r="90" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="90" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
@@ -2993,9 +2901,8 @@
       <c r="X90" s="1"/>
       <c r="Y90" s="1"/>
       <c r="Z90" s="1"/>
-      <c r="AA90" s="1"/>
-    </row>
-    <row r="91" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="91" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
@@ -3022,9 +2929,8 @@
       <c r="X91" s="1"/>
       <c r="Y91" s="1"/>
       <c r="Z91" s="1"/>
-      <c r="AA91" s="1"/>
-    </row>
-    <row r="92" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
@@ -3051,9 +2957,8 @@
       <c r="X92" s="1"/>
       <c r="Y92" s="1"/>
       <c r="Z92" s="1"/>
-      <c r="AA92" s="1"/>
-    </row>
-    <row r="93" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="93" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
@@ -3080,9 +2985,8 @@
       <c r="X93" s="1"/>
       <c r="Y93" s="1"/>
       <c r="Z93" s="1"/>
-      <c r="AA93" s="1"/>
-    </row>
-    <row r="94" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="94" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
@@ -3109,9 +3013,8 @@
       <c r="X94" s="1"/>
       <c r="Y94" s="1"/>
       <c r="Z94" s="1"/>
-      <c r="AA94" s="1"/>
-    </row>
-    <row r="95" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="95" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
@@ -3138,9 +3041,8 @@
       <c r="X95" s="1"/>
       <c r="Y95" s="1"/>
       <c r="Z95" s="1"/>
-      <c r="AA95" s="1"/>
-    </row>
-    <row r="96" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
@@ -3167,9 +3069,8 @@
       <c r="X96" s="1"/>
       <c r="Y96" s="1"/>
       <c r="Z96" s="1"/>
-      <c r="AA96" s="1"/>
-    </row>
-    <row r="97" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="97" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
@@ -3196,9 +3097,8 @@
       <c r="X97" s="1"/>
       <c r="Y97" s="1"/>
       <c r="Z97" s="1"/>
-      <c r="AA97" s="1"/>
-    </row>
-    <row r="98" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="98" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
@@ -3225,9 +3125,8 @@
       <c r="X98" s="1"/>
       <c r="Y98" s="1"/>
       <c r="Z98" s="1"/>
-      <c r="AA98" s="1"/>
-    </row>
-    <row r="99" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="99" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="1"/>
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
@@ -3254,9 +3153,8 @@
       <c r="X99" s="1"/>
       <c r="Y99" s="1"/>
       <c r="Z99" s="1"/>
-      <c r="AA99" s="1"/>
-    </row>
-    <row r="100" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="100" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="1"/>
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
@@ -3283,9 +3181,8 @@
       <c r="X100" s="1"/>
       <c r="Y100" s="1"/>
       <c r="Z100" s="1"/>
-      <c r="AA100" s="1"/>
-    </row>
-    <row r="101" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="101" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="1"/>
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
@@ -3312,9 +3209,8 @@
       <c r="X101" s="1"/>
       <c r="Y101" s="1"/>
       <c r="Z101" s="1"/>
-      <c r="AA101" s="1"/>
-    </row>
-    <row r="102" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="102" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="1"/>
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
@@ -3341,9 +3237,8 @@
       <c r="X102" s="1"/>
       <c r="Y102" s="1"/>
       <c r="Z102" s="1"/>
-      <c r="AA102" s="1"/>
-    </row>
-    <row r="103" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="103" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
@@ -3370,9 +3265,8 @@
       <c r="X103" s="1"/>
       <c r="Y103" s="1"/>
       <c r="Z103" s="1"/>
-      <c r="AA103" s="1"/>
-    </row>
-    <row r="104" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="104" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -3399,9 +3293,8 @@
       <c r="X104" s="1"/>
       <c r="Y104" s="1"/>
       <c r="Z104" s="1"/>
-      <c r="AA104" s="1"/>
-    </row>
-    <row r="105" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="105" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="1"/>
       <c r="B105" s="1"/>
       <c r="C105" s="1"/>
@@ -3428,9 +3321,8 @@
       <c r="X105" s="1"/>
       <c r="Y105" s="1"/>
       <c r="Z105" s="1"/>
-      <c r="AA105" s="1"/>
-    </row>
-    <row r="106" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="106" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="1"/>
       <c r="B106" s="1"/>
       <c r="C106" s="1"/>
@@ -3457,9 +3349,8 @@
       <c r="X106" s="1"/>
       <c r="Y106" s="1"/>
       <c r="Z106" s="1"/>
-      <c r="AA106" s="1"/>
-    </row>
-    <row r="107" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="107" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="1"/>
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
@@ -3486,9 +3377,8 @@
       <c r="X107" s="1"/>
       <c r="Y107" s="1"/>
       <c r="Z107" s="1"/>
-      <c r="AA107" s="1"/>
-    </row>
-    <row r="108" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="108" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="1"/>
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
@@ -3515,9 +3405,8 @@
       <c r="X108" s="1"/>
       <c r="Y108" s="1"/>
       <c r="Z108" s="1"/>
-      <c r="AA108" s="1"/>
-    </row>
-    <row r="109" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="109" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="1"/>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
@@ -3544,9 +3433,8 @@
       <c r="X109" s="1"/>
       <c r="Y109" s="1"/>
       <c r="Z109" s="1"/>
-      <c r="AA109" s="1"/>
-    </row>
-    <row r="110" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="110" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -3573,9 +3461,8 @@
       <c r="X110" s="1"/>
       <c r="Y110" s="1"/>
       <c r="Z110" s="1"/>
-      <c r="AA110" s="1"/>
-    </row>
-    <row r="111" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="111" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="1"/>
       <c r="B111" s="1"/>
       <c r="C111" s="1"/>
@@ -3602,9 +3489,8 @@
       <c r="X111" s="1"/>
       <c r="Y111" s="1"/>
       <c r="Z111" s="1"/>
-      <c r="AA111" s="1"/>
-    </row>
-    <row r="112" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="112" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="1"/>
       <c r="B112" s="1"/>
       <c r="C112" s="1"/>
@@ -3631,9 +3517,8 @@
       <c r="X112" s="1"/>
       <c r="Y112" s="1"/>
       <c r="Z112" s="1"/>
-      <c r="AA112" s="1"/>
-    </row>
-    <row r="113" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="113" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="1"/>
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
@@ -3660,9 +3545,8 @@
       <c r="X113" s="1"/>
       <c r="Y113" s="1"/>
       <c r="Z113" s="1"/>
-      <c r="AA113" s="1"/>
-    </row>
-    <row r="114" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="114" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
@@ -3689,9 +3573,8 @@
       <c r="X114" s="1"/>
       <c r="Y114" s="1"/>
       <c r="Z114" s="1"/>
-      <c r="AA114" s="1"/>
-    </row>
-    <row r="115" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="115" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
@@ -3718,9 +3601,8 @@
       <c r="X115" s="1"/>
       <c r="Y115" s="1"/>
       <c r="Z115" s="1"/>
-      <c r="AA115" s="1"/>
-    </row>
-    <row r="116" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="116" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
@@ -3747,9 +3629,8 @@
       <c r="X116" s="1"/>
       <c r="Y116" s="1"/>
       <c r="Z116" s="1"/>
-      <c r="AA116" s="1"/>
-    </row>
-    <row r="117" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="117" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="1"/>
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
@@ -3776,9 +3657,8 @@
       <c r="X117" s="1"/>
       <c r="Y117" s="1"/>
       <c r="Z117" s="1"/>
-      <c r="AA117" s="1"/>
-    </row>
-    <row r="118" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="118" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="1"/>
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
@@ -3805,9 +3685,8 @@
       <c r="X118" s="1"/>
       <c r="Y118" s="1"/>
       <c r="Z118" s="1"/>
-      <c r="AA118" s="1"/>
-    </row>
-    <row r="119" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="119" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="1"/>
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
@@ -3834,9 +3713,8 @@
       <c r="X119" s="1"/>
       <c r="Y119" s="1"/>
       <c r="Z119" s="1"/>
-      <c r="AA119" s="1"/>
-    </row>
-    <row r="120" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="120" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="1"/>
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
@@ -3863,9 +3741,8 @@
       <c r="X120" s="1"/>
       <c r="Y120" s="1"/>
       <c r="Z120" s="1"/>
-      <c r="AA120" s="1"/>
-    </row>
-    <row r="121" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="121" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="1"/>
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
@@ -3892,9 +3769,8 @@
       <c r="X121" s="1"/>
       <c r="Y121" s="1"/>
       <c r="Z121" s="1"/>
-      <c r="AA121" s="1"/>
-    </row>
-    <row r="122" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="122" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
@@ -3921,9 +3797,8 @@
       <c r="X122" s="1"/>
       <c r="Y122" s="1"/>
       <c r="Z122" s="1"/>
-      <c r="AA122" s="1"/>
-    </row>
-    <row r="123" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="123" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="1"/>
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
@@ -3950,9 +3825,8 @@
       <c r="X123" s="1"/>
       <c r="Y123" s="1"/>
       <c r="Z123" s="1"/>
-      <c r="AA123" s="1"/>
-    </row>
-    <row r="124" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="124" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1"/>
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
@@ -3979,9 +3853,8 @@
       <c r="X124" s="1"/>
       <c r="Y124" s="1"/>
       <c r="Z124" s="1"/>
-      <c r="AA124" s="1"/>
-    </row>
-    <row r="125" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="125" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="1"/>
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
@@ -4008,9 +3881,8 @@
       <c r="X125" s="1"/>
       <c r="Y125" s="1"/>
       <c r="Z125" s="1"/>
-      <c r="AA125" s="1"/>
-    </row>
-    <row r="126" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="126" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="1"/>
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
@@ -4037,9 +3909,8 @@
       <c r="X126" s="1"/>
       <c r="Y126" s="1"/>
       <c r="Z126" s="1"/>
-      <c r="AA126" s="1"/>
-    </row>
-    <row r="127" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="127" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="1"/>
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
@@ -4066,9 +3937,8 @@
       <c r="X127" s="1"/>
       <c r="Y127" s="1"/>
       <c r="Z127" s="1"/>
-      <c r="AA127" s="1"/>
-    </row>
-    <row r="128" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="128" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="1"/>
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
@@ -4095,9 +3965,8 @@
       <c r="X128" s="1"/>
       <c r="Y128" s="1"/>
       <c r="Z128" s="1"/>
-      <c r="AA128" s="1"/>
-    </row>
-    <row r="129" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="129" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="1"/>
       <c r="B129" s="1"/>
       <c r="C129" s="1"/>
@@ -4124,9 +3993,8 @@
       <c r="X129" s="1"/>
       <c r="Y129" s="1"/>
       <c r="Z129" s="1"/>
-      <c r="AA129" s="1"/>
-    </row>
-    <row r="130" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="130" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="1"/>
       <c r="B130" s="1"/>
       <c r="C130" s="1"/>
@@ -4153,9 +4021,8 @@
       <c r="X130" s="1"/>
       <c r="Y130" s="1"/>
       <c r="Z130" s="1"/>
-      <c r="AA130" s="1"/>
-    </row>
-    <row r="131" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="131" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="1"/>
       <c r="B131" s="1"/>
       <c r="C131" s="1"/>
@@ -4182,9 +4049,8 @@
       <c r="X131" s="1"/>
       <c r="Y131" s="1"/>
       <c r="Z131" s="1"/>
-      <c r="AA131" s="1"/>
-    </row>
-    <row r="132" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="132" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="1"/>
       <c r="B132" s="1"/>
       <c r="C132" s="1"/>
@@ -4211,9 +4077,8 @@
       <c r="X132" s="1"/>
       <c r="Y132" s="1"/>
       <c r="Z132" s="1"/>
-      <c r="AA132" s="1"/>
-    </row>
-    <row r="133" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="133" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="1"/>
       <c r="B133" s="1"/>
       <c r="C133" s="1"/>
@@ -4240,9 +4105,8 @@
       <c r="X133" s="1"/>
       <c r="Y133" s="1"/>
       <c r="Z133" s="1"/>
-      <c r="AA133" s="1"/>
-    </row>
-    <row r="134" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="134" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="1"/>
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
@@ -4269,9 +4133,8 @@
       <c r="X134" s="1"/>
       <c r="Y134" s="1"/>
       <c r="Z134" s="1"/>
-      <c r="AA134" s="1"/>
-    </row>
-    <row r="135" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="135" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="1"/>
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
@@ -4298,9 +4161,8 @@
       <c r="X135" s="1"/>
       <c r="Y135" s="1"/>
       <c r="Z135" s="1"/>
-      <c r="AA135" s="1"/>
-    </row>
-    <row r="136" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="136" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="1"/>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
@@ -4327,9 +4189,8 @@
       <c r="X136" s="1"/>
       <c r="Y136" s="1"/>
       <c r="Z136" s="1"/>
-      <c r="AA136" s="1"/>
-    </row>
-    <row r="137" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="137" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="1"/>
       <c r="B137" s="1"/>
       <c r="C137" s="1"/>
@@ -4356,9 +4217,8 @@
       <c r="X137" s="1"/>
       <c r="Y137" s="1"/>
       <c r="Z137" s="1"/>
-      <c r="AA137" s="1"/>
-    </row>
-    <row r="138" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="138" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="1"/>
       <c r="B138" s="1"/>
       <c r="C138" s="1"/>
@@ -4385,9 +4245,8 @@
       <c r="X138" s="1"/>
       <c r="Y138" s="1"/>
       <c r="Z138" s="1"/>
-      <c r="AA138" s="1"/>
-    </row>
-    <row r="139" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="139" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="1"/>
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
@@ -4414,9 +4273,8 @@
       <c r="X139" s="1"/>
       <c r="Y139" s="1"/>
       <c r="Z139" s="1"/>
-      <c r="AA139" s="1"/>
-    </row>
-    <row r="140" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="140" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="1"/>
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
@@ -4443,9 +4301,8 @@
       <c r="X140" s="1"/>
       <c r="Y140" s="1"/>
       <c r="Z140" s="1"/>
-      <c r="AA140" s="1"/>
-    </row>
-    <row r="141" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="141" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="1"/>
       <c r="B141" s="1"/>
       <c r="C141" s="1"/>
@@ -4472,9 +4329,8 @@
       <c r="X141" s="1"/>
       <c r="Y141" s="1"/>
       <c r="Z141" s="1"/>
-      <c r="AA141" s="1"/>
-    </row>
-    <row r="142" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="142" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
@@ -4501,9 +4357,8 @@
       <c r="X142" s="1"/>
       <c r="Y142" s="1"/>
       <c r="Z142" s="1"/>
-      <c r="AA142" s="1"/>
-    </row>
-    <row r="143" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="143" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="1"/>
       <c r="B143" s="1"/>
       <c r="C143" s="1"/>
@@ -4530,9 +4385,8 @@
       <c r="X143" s="1"/>
       <c r="Y143" s="1"/>
       <c r="Z143" s="1"/>
-      <c r="AA143" s="1"/>
-    </row>
-    <row r="144" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="144" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="1"/>
       <c r="B144" s="1"/>
       <c r="C144" s="1"/>
@@ -4559,9 +4413,8 @@
       <c r="X144" s="1"/>
       <c r="Y144" s="1"/>
       <c r="Z144" s="1"/>
-      <c r="AA144" s="1"/>
-    </row>
-    <row r="145" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="145" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="1"/>
       <c r="B145" s="1"/>
       <c r="C145" s="1"/>
@@ -4588,9 +4441,8 @@
       <c r="X145" s="1"/>
       <c r="Y145" s="1"/>
       <c r="Z145" s="1"/>
-      <c r="AA145" s="1"/>
-    </row>
-    <row r="146" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="146" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="1"/>
       <c r="B146" s="1"/>
       <c r="C146" s="1"/>
@@ -4617,9 +4469,8 @@
       <c r="X146" s="1"/>
       <c r="Y146" s="1"/>
       <c r="Z146" s="1"/>
-      <c r="AA146" s="1"/>
-    </row>
-    <row r="147" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="147" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="1"/>
       <c r="B147" s="1"/>
       <c r="C147" s="1"/>
@@ -4646,9 +4497,8 @@
       <c r="X147" s="1"/>
       <c r="Y147" s="1"/>
       <c r="Z147" s="1"/>
-      <c r="AA147" s="1"/>
-    </row>
-    <row r="148" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="148" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
@@ -4675,9 +4525,8 @@
       <c r="X148" s="1"/>
       <c r="Y148" s="1"/>
       <c r="Z148" s="1"/>
-      <c r="AA148" s="1"/>
-    </row>
-    <row r="149" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="149" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="1"/>
       <c r="B149" s="1"/>
       <c r="C149" s="1"/>
@@ -4704,9 +4553,8 @@
       <c r="X149" s="1"/>
       <c r="Y149" s="1"/>
       <c r="Z149" s="1"/>
-      <c r="AA149" s="1"/>
-    </row>
-    <row r="150" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="150" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="1"/>
       <c r="B150" s="1"/>
       <c r="C150" s="1"/>
@@ -4733,9 +4581,8 @@
       <c r="X150" s="1"/>
       <c r="Y150" s="1"/>
       <c r="Z150" s="1"/>
-      <c r="AA150" s="1"/>
-    </row>
-    <row r="151" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="151" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="1"/>
       <c r="B151" s="1"/>
       <c r="C151" s="1"/>
@@ -4762,9 +4609,8 @@
       <c r="X151" s="1"/>
       <c r="Y151" s="1"/>
       <c r="Z151" s="1"/>
-      <c r="AA151" s="1"/>
-    </row>
-    <row r="152" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="152" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="1"/>
       <c r="B152" s="1"/>
       <c r="C152" s="1"/>
@@ -4791,9 +4637,8 @@
       <c r="X152" s="1"/>
       <c r="Y152" s="1"/>
       <c r="Z152" s="1"/>
-      <c r="AA152" s="1"/>
-    </row>
-    <row r="153" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="153" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="1"/>
       <c r="B153" s="1"/>
       <c r="C153" s="1"/>
@@ -4820,9 +4665,8 @@
       <c r="X153" s="1"/>
       <c r="Y153" s="1"/>
       <c r="Z153" s="1"/>
-      <c r="AA153" s="1"/>
-    </row>
-    <row r="154" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="154" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
@@ -4849,9 +4693,8 @@
       <c r="X154" s="1"/>
       <c r="Y154" s="1"/>
       <c r="Z154" s="1"/>
-      <c r="AA154" s="1"/>
-    </row>
-    <row r="155" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="155" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="1"/>
       <c r="B155" s="1"/>
       <c r="C155" s="1"/>
@@ -4878,9 +4721,8 @@
       <c r="X155" s="1"/>
       <c r="Y155" s="1"/>
       <c r="Z155" s="1"/>
-      <c r="AA155" s="1"/>
-    </row>
-    <row r="156" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="156" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="1"/>
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
@@ -4907,9 +4749,8 @@
       <c r="X156" s="1"/>
       <c r="Y156" s="1"/>
       <c r="Z156" s="1"/>
-      <c r="AA156" s="1"/>
-    </row>
-    <row r="157" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="157" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="1"/>
       <c r="B157" s="1"/>
       <c r="C157" s="1"/>
@@ -4936,9 +4777,8 @@
       <c r="X157" s="1"/>
       <c r="Y157" s="1"/>
       <c r="Z157" s="1"/>
-      <c r="AA157" s="1"/>
-    </row>
-    <row r="158" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="158" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="1"/>
       <c r="B158" s="1"/>
       <c r="C158" s="1"/>
@@ -4965,9 +4805,8 @@
       <c r="X158" s="1"/>
       <c r="Y158" s="1"/>
       <c r="Z158" s="1"/>
-      <c r="AA158" s="1"/>
-    </row>
-    <row r="159" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="159" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="1"/>
       <c r="B159" s="1"/>
       <c r="C159" s="1"/>
@@ -4994,9 +4833,8 @@
       <c r="X159" s="1"/>
       <c r="Y159" s="1"/>
       <c r="Z159" s="1"/>
-      <c r="AA159" s="1"/>
-    </row>
-    <row r="160" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="160" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="1"/>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
@@ -5023,9 +4861,8 @@
       <c r="X160" s="1"/>
       <c r="Y160" s="1"/>
       <c r="Z160" s="1"/>
-      <c r="AA160" s="1"/>
-    </row>
-    <row r="161" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="161" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="1"/>
       <c r="B161" s="1"/>
       <c r="C161" s="1"/>
@@ -5052,9 +4889,8 @@
       <c r="X161" s="1"/>
       <c r="Y161" s="1"/>
       <c r="Z161" s="1"/>
-      <c r="AA161" s="1"/>
-    </row>
-    <row r="162" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="162" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="1"/>
       <c r="B162" s="1"/>
       <c r="C162" s="1"/>
@@ -5081,9 +4917,8 @@
       <c r="X162" s="1"/>
       <c r="Y162" s="1"/>
       <c r="Z162" s="1"/>
-      <c r="AA162" s="1"/>
-    </row>
-    <row r="163" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="163" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="1"/>
       <c r="B163" s="1"/>
       <c r="C163" s="1"/>
@@ -5110,9 +4945,8 @@
       <c r="X163" s="1"/>
       <c r="Y163" s="1"/>
       <c r="Z163" s="1"/>
-      <c r="AA163" s="1"/>
-    </row>
-    <row r="164" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="164" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="1"/>
       <c r="B164" s="1"/>
       <c r="C164" s="1"/>
@@ -5139,9 +4973,8 @@
       <c r="X164" s="1"/>
       <c r="Y164" s="1"/>
       <c r="Z164" s="1"/>
-      <c r="AA164" s="1"/>
-    </row>
-    <row r="165" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="165" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="1"/>
       <c r="B165" s="1"/>
       <c r="C165" s="1"/>
@@ -5168,9 +5001,8 @@
       <c r="X165" s="1"/>
       <c r="Y165" s="1"/>
       <c r="Z165" s="1"/>
-      <c r="AA165" s="1"/>
-    </row>
-    <row r="166" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="166" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="1"/>
       <c r="B166" s="1"/>
       <c r="C166" s="1"/>
@@ -5197,9 +5029,8 @@
       <c r="X166" s="1"/>
       <c r="Y166" s="1"/>
       <c r="Z166" s="1"/>
-      <c r="AA166" s="1"/>
-    </row>
-    <row r="167" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="167" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="1"/>
       <c r="B167" s="1"/>
       <c r="C167" s="1"/>
@@ -5226,9 +5057,8 @@
       <c r="X167" s="1"/>
       <c r="Y167" s="1"/>
       <c r="Z167" s="1"/>
-      <c r="AA167" s="1"/>
-    </row>
-    <row r="168" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="168" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="1"/>
       <c r="B168" s="1"/>
       <c r="C168" s="1"/>
@@ -5255,9 +5085,8 @@
       <c r="X168" s="1"/>
       <c r="Y168" s="1"/>
       <c r="Z168" s="1"/>
-      <c r="AA168" s="1"/>
-    </row>
-    <row r="169" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="169" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="1"/>
       <c r="B169" s="1"/>
       <c r="C169" s="1"/>
@@ -5284,9 +5113,8 @@
       <c r="X169" s="1"/>
       <c r="Y169" s="1"/>
       <c r="Z169" s="1"/>
-      <c r="AA169" s="1"/>
-    </row>
-    <row r="170" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="170" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="1"/>
       <c r="B170" s="1"/>
       <c r="C170" s="1"/>
@@ -5313,9 +5141,8 @@
       <c r="X170" s="1"/>
       <c r="Y170" s="1"/>
       <c r="Z170" s="1"/>
-      <c r="AA170" s="1"/>
-    </row>
-    <row r="171" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="171" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="1"/>
       <c r="B171" s="1"/>
       <c r="C171" s="1"/>
@@ -5342,9 +5169,8 @@
       <c r="X171" s="1"/>
       <c r="Y171" s="1"/>
       <c r="Z171" s="1"/>
-      <c r="AA171" s="1"/>
-    </row>
-    <row r="172" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="172" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="1"/>
       <c r="B172" s="1"/>
       <c r="C172" s="1"/>
@@ -5371,9 +5197,8 @@
       <c r="X172" s="1"/>
       <c r="Y172" s="1"/>
       <c r="Z172" s="1"/>
-      <c r="AA172" s="1"/>
-    </row>
-    <row r="173" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="173" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="1"/>
       <c r="B173" s="1"/>
       <c r="C173" s="1"/>
@@ -5400,9 +5225,8 @@
       <c r="X173" s="1"/>
       <c r="Y173" s="1"/>
       <c r="Z173" s="1"/>
-      <c r="AA173" s="1"/>
-    </row>
-    <row r="174" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="174" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="1"/>
       <c r="B174" s="1"/>
       <c r="C174" s="1"/>
@@ -5429,9 +5253,8 @@
       <c r="X174" s="1"/>
       <c r="Y174" s="1"/>
       <c r="Z174" s="1"/>
-      <c r="AA174" s="1"/>
-    </row>
-    <row r="175" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="175" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="1"/>
       <c r="B175" s="1"/>
       <c r="C175" s="1"/>
@@ -5458,9 +5281,8 @@
       <c r="X175" s="1"/>
       <c r="Y175" s="1"/>
       <c r="Z175" s="1"/>
-      <c r="AA175" s="1"/>
-    </row>
-    <row r="176" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="176" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="1"/>
       <c r="B176" s="1"/>
       <c r="C176" s="1"/>
@@ -5487,9 +5309,8 @@
       <c r="X176" s="1"/>
       <c r="Y176" s="1"/>
       <c r="Z176" s="1"/>
-      <c r="AA176" s="1"/>
-    </row>
-    <row r="177" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="177" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="1"/>
       <c r="B177" s="1"/>
       <c r="C177" s="1"/>
@@ -5516,9 +5337,8 @@
       <c r="X177" s="1"/>
       <c r="Y177" s="1"/>
       <c r="Z177" s="1"/>
-      <c r="AA177" s="1"/>
-    </row>
-    <row r="178" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="178" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="1"/>
       <c r="B178" s="1"/>
       <c r="C178" s="1"/>
@@ -5545,9 +5365,8 @@
       <c r="X178" s="1"/>
       <c r="Y178" s="1"/>
       <c r="Z178" s="1"/>
-      <c r="AA178" s="1"/>
-    </row>
-    <row r="179" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="179" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="1"/>
       <c r="B179" s="1"/>
       <c r="C179" s="1"/>
@@ -5574,9 +5393,8 @@
       <c r="X179" s="1"/>
       <c r="Y179" s="1"/>
       <c r="Z179" s="1"/>
-      <c r="AA179" s="1"/>
-    </row>
-    <row r="180" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="180" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="1"/>
       <c r="B180" s="1"/>
       <c r="C180" s="1"/>
@@ -5603,9 +5421,8 @@
       <c r="X180" s="1"/>
       <c r="Y180" s="1"/>
       <c r="Z180" s="1"/>
-      <c r="AA180" s="1"/>
-    </row>
-    <row r="181" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="181" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="1"/>
       <c r="B181" s="1"/>
       <c r="C181" s="1"/>
@@ -5632,9 +5449,8 @@
       <c r="X181" s="1"/>
       <c r="Y181" s="1"/>
       <c r="Z181" s="1"/>
-      <c r="AA181" s="1"/>
-    </row>
-    <row r="182" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="182" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="1"/>
       <c r="B182" s="1"/>
       <c r="C182" s="1"/>
@@ -5661,9 +5477,8 @@
       <c r="X182" s="1"/>
       <c r="Y182" s="1"/>
       <c r="Z182" s="1"/>
-      <c r="AA182" s="1"/>
-    </row>
-    <row r="183" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="183" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="1"/>
       <c r="B183" s="1"/>
       <c r="C183" s="1"/>
@@ -5690,9 +5505,8 @@
       <c r="X183" s="1"/>
       <c r="Y183" s="1"/>
       <c r="Z183" s="1"/>
-      <c r="AA183" s="1"/>
-    </row>
-    <row r="184" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="184" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="1"/>
       <c r="B184" s="1"/>
       <c r="C184" s="1"/>
@@ -5719,9 +5533,8 @@
       <c r="X184" s="1"/>
       <c r="Y184" s="1"/>
       <c r="Z184" s="1"/>
-      <c r="AA184" s="1"/>
-    </row>
-    <row r="185" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="185" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="1"/>
       <c r="B185" s="1"/>
       <c r="C185" s="1"/>
@@ -5748,9 +5561,8 @@
       <c r="X185" s="1"/>
       <c r="Y185" s="1"/>
       <c r="Z185" s="1"/>
-      <c r="AA185" s="1"/>
-    </row>
-    <row r="186" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="186" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="1"/>
       <c r="B186" s="1"/>
       <c r="C186" s="1"/>
@@ -5777,9 +5589,8 @@
       <c r="X186" s="1"/>
       <c r="Y186" s="1"/>
       <c r="Z186" s="1"/>
-      <c r="AA186" s="1"/>
-    </row>
-    <row r="187" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="187" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="1"/>
       <c r="B187" s="1"/>
       <c r="C187" s="1"/>
@@ -5806,9 +5617,8 @@
       <c r="X187" s="1"/>
       <c r="Y187" s="1"/>
       <c r="Z187" s="1"/>
-      <c r="AA187" s="1"/>
-    </row>
-    <row r="188" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="188" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="1"/>
       <c r="B188" s="1"/>
       <c r="C188" s="1"/>
@@ -5835,9 +5645,8 @@
       <c r="X188" s="1"/>
       <c r="Y188" s="1"/>
       <c r="Z188" s="1"/>
-      <c r="AA188" s="1"/>
-    </row>
-    <row r="189" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="189" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="1"/>
       <c r="B189" s="1"/>
       <c r="C189" s="1"/>
@@ -5864,9 +5673,8 @@
       <c r="X189" s="1"/>
       <c r="Y189" s="1"/>
       <c r="Z189" s="1"/>
-      <c r="AA189" s="1"/>
-    </row>
-    <row r="190" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="190" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="1"/>
       <c r="B190" s="1"/>
       <c r="C190" s="1"/>
@@ -5893,9 +5701,8 @@
       <c r="X190" s="1"/>
       <c r="Y190" s="1"/>
       <c r="Z190" s="1"/>
-      <c r="AA190" s="1"/>
-    </row>
-    <row r="191" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="191" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="1"/>
       <c r="B191" s="1"/>
       <c r="C191" s="1"/>
@@ -5922,9 +5729,8 @@
       <c r="X191" s="1"/>
       <c r="Y191" s="1"/>
       <c r="Z191" s="1"/>
-      <c r="AA191" s="1"/>
-    </row>
-    <row r="192" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="192" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="1"/>
       <c r="B192" s="1"/>
       <c r="C192" s="1"/>
@@ -5951,9 +5757,8 @@
       <c r="X192" s="1"/>
       <c r="Y192" s="1"/>
       <c r="Z192" s="1"/>
-      <c r="AA192" s="1"/>
-    </row>
-    <row r="193" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="193" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="1"/>
       <c r="B193" s="1"/>
       <c r="C193" s="1"/>
@@ -5980,9 +5785,8 @@
       <c r="X193" s="1"/>
       <c r="Y193" s="1"/>
       <c r="Z193" s="1"/>
-      <c r="AA193" s="1"/>
-    </row>
-    <row r="194" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="194" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="1"/>
       <c r="B194" s="1"/>
       <c r="C194" s="1"/>
@@ -6009,9 +5813,8 @@
       <c r="X194" s="1"/>
       <c r="Y194" s="1"/>
       <c r="Z194" s="1"/>
-      <c r="AA194" s="1"/>
-    </row>
-    <row r="195" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="195" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="1"/>
       <c r="B195" s="1"/>
       <c r="C195" s="1"/>
@@ -6038,9 +5841,8 @@
       <c r="X195" s="1"/>
       <c r="Y195" s="1"/>
       <c r="Z195" s="1"/>
-      <c r="AA195" s="1"/>
-    </row>
-    <row r="196" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="196" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="1"/>
       <c r="B196" s="1"/>
       <c r="C196" s="1"/>
@@ -6067,9 +5869,8 @@
       <c r="X196" s="1"/>
       <c r="Y196" s="1"/>
       <c r="Z196" s="1"/>
-      <c r="AA196" s="1"/>
-    </row>
-    <row r="197" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="197" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="1"/>
       <c r="B197" s="1"/>
       <c r="C197" s="1"/>
@@ -6096,9 +5897,8 @@
       <c r="X197" s="1"/>
       <c r="Y197" s="1"/>
       <c r="Z197" s="1"/>
-      <c r="AA197" s="1"/>
-    </row>
-    <row r="198" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="198" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="1"/>
       <c r="B198" s="1"/>
       <c r="C198" s="1"/>
@@ -6125,9 +5925,8 @@
       <c r="X198" s="1"/>
       <c r="Y198" s="1"/>
       <c r="Z198" s="1"/>
-      <c r="AA198" s="1"/>
-    </row>
-    <row r="199" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="199" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="1"/>
       <c r="B199" s="1"/>
       <c r="C199" s="1"/>
@@ -6154,9 +5953,8 @@
       <c r="X199" s="1"/>
       <c r="Y199" s="1"/>
       <c r="Z199" s="1"/>
-      <c r="AA199" s="1"/>
-    </row>
-    <row r="200" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="200" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="1"/>
       <c r="B200" s="1"/>
       <c r="C200" s="1"/>
@@ -6183,9 +5981,8 @@
       <c r="X200" s="1"/>
       <c r="Y200" s="1"/>
       <c r="Z200" s="1"/>
-      <c r="AA200" s="1"/>
-    </row>
-    <row r="201" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="201" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="1"/>
       <c r="B201" s="1"/>
       <c r="C201" s="1"/>
@@ -6212,9 +6009,8 @@
       <c r="X201" s="1"/>
       <c r="Y201" s="1"/>
       <c r="Z201" s="1"/>
-      <c r="AA201" s="1"/>
-    </row>
-    <row r="202" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="202" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A202" s="1"/>
       <c r="B202" s="1"/>
       <c r="C202" s="1"/>
@@ -6241,9 +6037,8 @@
       <c r="X202" s="1"/>
       <c r="Y202" s="1"/>
       <c r="Z202" s="1"/>
-      <c r="AA202" s="1"/>
-    </row>
-    <row r="203" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="203" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A203" s="1"/>
       <c r="B203" s="1"/>
       <c r="C203" s="1"/>
@@ -6270,9 +6065,8 @@
       <c r="X203" s="1"/>
       <c r="Y203" s="1"/>
       <c r="Z203" s="1"/>
-      <c r="AA203" s="1"/>
-    </row>
-    <row r="204" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="204" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="1"/>
       <c r="B204" s="1"/>
       <c r="C204" s="1"/>
@@ -6299,9 +6093,8 @@
       <c r="X204" s="1"/>
       <c r="Y204" s="1"/>
       <c r="Z204" s="1"/>
-      <c r="AA204" s="1"/>
-    </row>
-    <row r="205" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="205" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="1"/>
       <c r="B205" s="1"/>
       <c r="C205" s="1"/>
@@ -6328,9 +6121,8 @@
       <c r="X205" s="1"/>
       <c r="Y205" s="1"/>
       <c r="Z205" s="1"/>
-      <c r="AA205" s="1"/>
-    </row>
-    <row r="206" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="206" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="1"/>
       <c r="B206" s="1"/>
       <c r="C206" s="1"/>
@@ -6357,9 +6149,8 @@
       <c r="X206" s="1"/>
       <c r="Y206" s="1"/>
       <c r="Z206" s="1"/>
-      <c r="AA206" s="1"/>
-    </row>
-    <row r="207" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="207" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="1"/>
       <c r="B207" s="1"/>
       <c r="C207" s="1"/>
@@ -6386,9 +6177,8 @@
       <c r="X207" s="1"/>
       <c r="Y207" s="1"/>
       <c r="Z207" s="1"/>
-      <c r="AA207" s="1"/>
-    </row>
-    <row r="208" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="208" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="1"/>
       <c r="B208" s="1"/>
       <c r="C208" s="1"/>
@@ -6415,9 +6205,8 @@
       <c r="X208" s="1"/>
       <c r="Y208" s="1"/>
       <c r="Z208" s="1"/>
-      <c r="AA208" s="1"/>
-    </row>
-    <row r="209" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="209" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A209" s="1"/>
       <c r="B209" s="1"/>
       <c r="C209" s="1"/>
@@ -6444,9 +6233,8 @@
       <c r="X209" s="1"/>
       <c r="Y209" s="1"/>
       <c r="Z209" s="1"/>
-      <c r="AA209" s="1"/>
-    </row>
-    <row r="210" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="210" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A210" s="1"/>
       <c r="B210" s="1"/>
       <c r="C210" s="1"/>
@@ -6473,9 +6261,8 @@
       <c r="X210" s="1"/>
       <c r="Y210" s="1"/>
       <c r="Z210" s="1"/>
-      <c r="AA210" s="1"/>
-    </row>
-    <row r="211" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="211" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A211" s="1"/>
       <c r="B211" s="1"/>
       <c r="C211" s="1"/>
@@ -6502,9 +6289,8 @@
       <c r="X211" s="1"/>
       <c r="Y211" s="1"/>
       <c r="Z211" s="1"/>
-      <c r="AA211" s="1"/>
-    </row>
-    <row r="212" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="212" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A212" s="1"/>
       <c r="B212" s="1"/>
       <c r="C212" s="1"/>
@@ -6531,9 +6317,8 @@
       <c r="X212" s="1"/>
       <c r="Y212" s="1"/>
       <c r="Z212" s="1"/>
-      <c r="AA212" s="1"/>
-    </row>
-    <row r="213" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="213" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A213" s="1"/>
       <c r="B213" s="1"/>
       <c r="C213" s="1"/>
@@ -6560,9 +6345,8 @@
       <c r="X213" s="1"/>
       <c r="Y213" s="1"/>
       <c r="Z213" s="1"/>
-      <c r="AA213" s="1"/>
-    </row>
-    <row r="214" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="214" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="1"/>
       <c r="B214" s="1"/>
       <c r="C214" s="1"/>
@@ -6589,9 +6373,8 @@
       <c r="X214" s="1"/>
       <c r="Y214" s="1"/>
       <c r="Z214" s="1"/>
-      <c r="AA214" s="1"/>
-    </row>
-    <row r="215" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="215" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A215" s="1"/>
       <c r="B215" s="1"/>
       <c r="C215" s="1"/>
@@ -6618,9 +6401,8 @@
       <c r="X215" s="1"/>
       <c r="Y215" s="1"/>
       <c r="Z215" s="1"/>
-      <c r="AA215" s="1"/>
-    </row>
-    <row r="216" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="216" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A216" s="1"/>
       <c r="B216" s="1"/>
       <c r="C216" s="1"/>
@@ -6647,9 +6429,8 @@
       <c r="X216" s="1"/>
       <c r="Y216" s="1"/>
       <c r="Z216" s="1"/>
-      <c r="AA216" s="1"/>
-    </row>
-    <row r="217" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="217" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A217" s="1"/>
       <c r="B217" s="1"/>
       <c r="C217" s="1"/>
@@ -6676,9 +6457,8 @@
       <c r="X217" s="1"/>
       <c r="Y217" s="1"/>
       <c r="Z217" s="1"/>
-      <c r="AA217" s="1"/>
-    </row>
-    <row r="218" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="218" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="1"/>
       <c r="B218" s="1"/>
       <c r="C218" s="1"/>
@@ -6705,9 +6485,8 @@
       <c r="X218" s="1"/>
       <c r="Y218" s="1"/>
       <c r="Z218" s="1"/>
-      <c r="AA218" s="1"/>
-    </row>
-    <row r="219" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="219" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A219" s="1"/>
       <c r="B219" s="1"/>
       <c r="C219" s="1"/>
@@ -6734,9 +6513,8 @@
       <c r="X219" s="1"/>
       <c r="Y219" s="1"/>
       <c r="Z219" s="1"/>
-      <c r="AA219" s="1"/>
-    </row>
-    <row r="220" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="220" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A220" s="1"/>
       <c r="B220" s="1"/>
       <c r="C220" s="1"/>
@@ -6763,12 +6541,11 @@
       <c r="X220" s="1"/>
       <c r="Y220" s="1"/>
       <c r="Z220" s="1"/>
-      <c r="AA220" s="1"/>
-    </row>
-    <row r="221" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="222" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="223" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="224" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    </row>
+    <row r="221" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="222" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="223" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="224" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>